<commit_message>
Download photos locally via export_changes.py
</commit_message>
<xml_diff>
--- a/WO_Changes.xlsx
+++ b/WO_Changes.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>["data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEA8ADwAAD/4TCmRXhpZgAASUkqAAgAAAAIAA8BAgAGAAAAbgAAABABAgAPAAAAdAAAABoBBQABAAAAhAAAABsBBQABAAAAjAAAACgBAwABAAAAAgAAADEBAgA1AAAAlAAAADIBAgAUAAAAygAAAGmHBAABAAAA3gAAAEIDAABDYW5vbgBDYW5vbiBFT1MgUjVtMgAA8AAAAAEAAADwAAAAAQAAAEFkb2JlIFBob3Rvc2hvcCBMaWdodHJvb20gQ2xhc3NpYyAxNS4xLjEgKE1hY2ludG9zaCkAADIwMjY6MDI6MTIgMDQ6MTE6MTAAIQCaggUAAQAAAHACAACdggUAAQAAAHgCAAAiiAMAAQAAAAEAAAAniAMAAQAAAKAAAAAwiAMAAQAAAAIAAAAyiAQAAQAAAKAAAAAAkAcABAAAADAyMzEDkAIAFAAAAIACAAAEkAIAFAAAAJQCAAAQkAIABwAAAKgCAAARkAIABwAAALACAAASkAIABwAAALgCAAABkgoAAQAAAMACAAACkgUAAQAAAMgCAAAEkgoAAQAAANACAAAFkgUAAQAAANgCAAAHkgMAAQAAAAUAAAAJkgMAAQAAAAAAAAAKkgUAAQAAAOACAACRkgIABAAAADEzMQCSkgIABAAAADEzMQABoAMAAQAAAAEAAAAOogUAAQAAAOgCAAAPogUAAQAAAPACAAAQogMAAQAAAAIAAAABpAMAAQAAAAAAAAACpAMAAQAAAAEAAAADpAMAAQAAAAEAAAAGpAMAAQAAAAAAAAAxpAIADQAAAPgCAAAypAUABAAAAAYDAAA0pAIADwAAACYDAAA1pAIACwAAADYDAAAAAAAAAQAAADwAAAAFAAAAAQAAADIwMjY6MDE6MjIgMTE6NTQ6MDUAMjAyNjowMToyMiAxMTo1NDowNQArMDY6MDAAAC0wNTowMAAALTA1OjAwAADLIVoAQEIPABDcRgBAQg8AAAAAAAEAAAADAAAAAQAAAFoAAAABAAAAAAB9AIsFAADAX1MAswMAADE1MjIwMjQwMDMwMQAAWgAAAAEAAABaAAAAAQAAAAAAAAAAAAAAAAAAAAAAAABUUy1FOTBtbSBmLzIuOAAAMDAwMDAwMDAwMAAABgADAQMAAQAAAAYAAAAaAQUAAQAAAJADAAAbAQUAAQAAAJgDAAAoAQMAAQAAAAIAAAABAgQAAQAAAKADAAACAgQAAQAAAP4sAAAAAAAASAAAAAEAAABIAAAAAQAAAP/Y/9sAhAAGBAQEBQQGBQUGCQYFBgkLCAYGCAsMCgoLCgoMEAwMDAwMDBAMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMAQcHBw0MDRgQEBgUDg4OFBQODg4OFBEMDAwMDBERDAwMDAwMEQwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAz/3QAEACD/7gAOQWRvYmUAZMAAAAAB/8AAEQgAqwEAAwARAAERAQIRAf/EAaIAAAAHAQEBAQEAAAAAAAAAAAQFAwIGAQAHCAkKCwEAAgIDAQEBAQEAAAAAAAAAAQACAwQFBgcICQoLEAACAQMDAgQCBgcDBAIGAnMBAgMRBAAFIRIxQVEGE2EicYEUMpGhBxWxQiPBUtHhMxZi8CRygvElQzRTkqKyY3PCNUQnk6OzNhdUZHTD0uIIJoMJChgZhJRFRqS0VtNVKBry4/PE1OT0ZXWFlaW1xdXl9WZ2hpamtsbW5vY3R1dnd4eXp7fH1+f3OEhYaHiImKi4yNjo+Ck5SVlpeYmZqbnJ2en5KjpKWmp6ipqqusra6voRAAICAQIDBQUEBQYECAMDbQEAAhEDBCESMUEFURNhIgZxgZEyobHwFMHR4SNCFVJicvEzJDRDghaSUyWiY7LCB3PSNeJEgxdUkwgJChgZJjZFGidkdFU38qOzwygp0+PzhJSktMTU5PRldYWVpbXF1eX1RlZmdoaWprbG1ub2R1dnd4eXp7fH1+f3OEhYaHiImKi4yNjo+DlJWWl5iZmpucnZ6fkqOkpaanqKmqq6ytrq+v/aAAwDAAABEQIRAD8APkTJKqquKrwMKuOKomU/uj/q/wAMtamLaavxOf8AKP68qb06iG2SYlEoMLFXUYqqAYqibYUST3GSixkx+Jf9Nm/1zkWfRH8dsLFSYEOp/wAofrwqn88lHOBCmJMVXq5xVUD4pb5jArg4riqoG3xVVR8VVkfFVdJMCoiN8UoqN8VRET7YFRKPiqqsvvgSqCTFXF8VU2fFX//QkarklXgYq2cKpH5t8xjQNIfUTAbgJJHH6Qbif3jca1IPTFWLS/nMihFOlN+8iVx++HRxX+XLOJhSXwfmjFAvI6YxDHr6v/NmQpnxI2L83oP+rY//ACMP/NGFFoyH82oWH/HOYfORv+qeFFoyL804G/48f+Sjf9U8VtEr+ZkZ6WBbv8Lsf+ZeNItFab+ZMd5EZLWx9aMkqXSQkAqaEH4OoPbJBBVNO1S6ubmVhbKhrUhnYdfmmCk8SHfzBrQkm3tkiid15Mj7KjEVJ5jwyNlnw7JV/wArFQqWM8VFO5+qz02Pb48u8Gfc0+NDvW3v5z2ltKyTzRiRdiBaXB/U5yBhIMhKJ6oI/ntYA/DNGf8AozuP+a8juyoJhp/5sajqLBbCOGQnpyt5UH4yZKMJFiTEMmjvPzIlhEsUOm8W3AJkr93LLfy0/Jr8eHmx7XPPfnjRrkW19BaRyMvKNhG7Iw/yW57075TOMomi2wIkLCVW35teaXv4IStpwkcK1InrQ/8APTIcTPhT0/mbr8fWG2b/AGLj/jfCwTjyh581PWdYayuLeFIxC8vKPkDVWUU3J/mwqziOY4qiElxVExPgVFxvilEI+BVdJMVVFkxVUEmBLvUxVaZMUP8A/9GTDJq7FWicVYV+a5/51Cb/AIzwf8nBipeS3xcPamQ1H1WDhvX4eOwHhhYqSOWap+gYqjIK4UJhBthVHwDChNrI8WHhhVUksrzTbltW0lPU50OoaepoJ1H7adlnUf8AIz7D/ssrS2y/Qryx1Zba5spqpPsrd1Kn4lZD0dSOLKw5LhQ8+/MjUdR0q1iewIU3NxKtwjglWVKkCldt/wCXBCwbHNM6MaLFdd806hHem0WC24JFAAxjdmNYUJ5ESKvfsuWDVSGzWdNG7S06vbXk0kmoBgW3Bt4gTX35zLgOe+f4+1PhVy/H2L4otBlkAWW6Vj0HoxD9cpyPGngLJ/LuuaZp0itHJdOi/smKEA/M865OOWipgXo8HnOWIPFJFPBLGnqGOZAhC0DfzHqDUZfg1sJ1w7gteTTkAkoPVvMFhrdgbW+QhTVreelCrjbkhPXwbMvJiExRcaGQxNhgMULQa5bxMQxWVaMOhHY5p5wMZUXZRmJCwySZcDFkP5Zj/nZpP+YWT/iaYQpeqAkYUKqSHAqLhkxSjInwKiFkxSqrJgVUWTFV4kxV3qe+KrTJir//0pLk1bxVa1cVYV+bI/506f8A4zwf8nBiryC7JLQf8YIqf8AMLFuEUocKoyE4oZB5Z0xdV1mz055DEt1II2lVeZUUJJC1FemSAtWV+aPJtnoenWF9a3st0l47IUmh9Fk4qG3HJj36HDIUSLumzLhlCuIVxBKrXti0pzZOVI8MKofyk/pfmHqsUXwQNFaytENlMjCQM/HpyIVanAOaeiSfmVF6lpZqRT/SJzSlMswiyWObkGIaV5J1TXDLfTzNbKLRr1JXhYpKkR4UUgqKtT7WarW6zwKJiZccxj/0/wDE5WPHxfLias/Ieo3GiXWqq0itbzx25smt5PWdpeJBUVr+104YZ6rhzxxUfXEz4/4fT/CgQuJl3K1z5Hv7TR7LVPVMqXnqEwpC/OJYjRmc1Pw/5VFxw6wZM08QBEsXD6v53GssdREv5ybyeTLrTNZsLGSdJ2ulglDBGChZnoAwqT23yrT9oRzYp5IiQ8Pjj/S/dspYjGQHeyrzM1/Lrd5b3fpfW44vQkMAZUNFqDRq78WC/wCxy3sTHEY4cHFwyPF6/qYayR9V9yWfVNUuYoLaaRmgtQwt0J2QOeTBfDk25zqhEui4wk81u8HmK2if7SulfpGajVCshdrpjeMMilQ5UzZD+Wi08yy/8wsn/E0xCvTypwocCcVRMLHAqLjfpgSiFfFVRZMUqiyYFXh8Vb54q0XxV//TkuTV2KuOKsL/ADZ/5Q2f/jPB/wAnBirx26PxQf8AGCL/AIiMLFdFhVFxHfFCaaXf3Vjdw3lpIYbmBg8Uq0qrDuKgjCrINT82eYdbSJNVv5LtICWiVwgCltiRxVeuFSXWjdMLFOLV+mFUJ5aen5iaqen+j2n/ADNyPVPRKvzFkK2dh+yTPcDp03G9Mu053LDOPSGZWuq6BB5NmbSJ4buG4NrZKY9zDZJIkUsklQGjWNPUaTkOKccxJTA5t4Hcnk1/pUfl6Jze26NcXUkrT+qnDm0bJGrS141NV4VP8uPELrqqKun0iW60/S4rq2WCOCFKllRJI2ZmlKVP7xDxTlwwCQJI6rTcOowXXm29nldYrS1vQqK5ChlhtYyh4Ehm/eM/Db7WII6JovLPrkz6hq9/c8uQu7xgz1qY/Xb0+v8AxWVzJ0pHHE9Las49Evcr23mK2DA1GdAJxdHwFJtTu4pfMMd4P7sFWNPBVzR60/vS7nSj92EbbeZNKu5RDG55tsAQcx2xmf5cqR5ll/5hJP8AiaYoZj5o856B5YtobrWbgwRXL+lCVjeUswUt9mMMeg64SoSO2/OLyDcB2ivpXEa85CLa4PFfFvg2X3OC00i4fzc8hHpqRp/xhl/5pxtaKKj/ADb8hD/paAfOKX/mnBaaKIT82vIDsFXVkLHYL6ctSfYcMbWm/wDlbn5fg0OsxD2KyD/jXFaZXp+p2t9ZwXlpKs1rcIssEyGqujiqsD4EYoRYlGKVwkwK7nir/9SSVyauBxV2KsM/NkA+Tpv+M8H/ABMYVLxy5PxxDwhj/wCIjFi3EdsKoqM4oRkLdMKplbnYYUJrat0woTe1fcYVQXl16fmDqp/4otf+ZmRHNPRKfzMPHT9N2pWe42Ip38Bk8XMoy8gt/KLT31XT9S06SLnb3NxHZ+sGPNEnUvMiLts6x8v9blmDlxiUxf8AD6nIiaiWY2vkfT7q5udEijk/QNlcSyoXldiRaKRxY9ePruv+xi4ZT4ZOWUuvDUfx/pm248AHmrQ+ULW80g6xfySxxaOiR6akJHE+sQONCCKEN6fCmVaaJEJz/in/ALxnm4eKITrQPKekSeZoNX1X1hLdTnTbGHZuPoxmjGv7RZZfjVvh5ZXlxnHpajt/EmJBypF+ZOhadpemXN3bXM7tq5ubhLaWgWOOPgnJBTkvNvi4kt9rNj2dEiML504uqIPFTyyF09LkG3zfg7OpIRtOcUbjeqN/xE5rNQfWXYYPoDGLLVHsZUmVF5qQRzO1cpZMn8v/AJr+ZtPvGvbTTILglGh3EgWhIJ3Fd/hx4lpX80+etX85QWttrGjC3itZDLE8DSAlmUrvVfA4k2kRSuztYbQTiz+tW/1mMxXARjR0NfhaqHbfFNNCxt0FBFcH7/8AmjAlY0Vuo+OK4HyNP1pihV0+/g069hvbVrmK5gJKOGjJ3BU7MhG6mmKkIa6uLS4uJJ5Xn9SZ2dmPp7sxJPYYq9f8ifmxGmi2+jW+mO7aRaQxNPJMB6gUcOVFU0rSuSYl6+tyaAkUJAxQrRzVxVWDYpf/1ZGDk1bGKuxVhn5smnk6Yj/f8H/E8VLxq6P7yL/jDH/xEYWLcZ2GFUTGcUIuFsKpjbN0woTW1bpiqawN0woS/RGZvPeq8G4MYbWjEVA/vO2Ac09Et/NEcNO0w1ILXFwSD0FPAdF+jJY+ZWfIMn/LPQ9U0XQpbpZ0himtkvZpN0ZJ54ysSGvNZOCvX7P8ua3VxybSgar6v6jk4qOxTezt/MFp5avw15Eour6SG2uwTwljLB5yQRVUd1lpw/ab4crySnHIJf5KQ9X87j/4lnCIlGv4ophf6V5yvvIENxCptwssd29ou4HpyLIkQYBW5ScV+2rcPs/t5i4808WY4pG4Trw/6PH/AMebJQEo8Q5j/er9T1HzHb+YtIaCNJobO6j9S0DIrrM/KScGlVKCNlblxRv8puWWxOWeKcJislGv97/pkUIyEhySL83oNajCyaiKQvZzwWp4lPslWJ4nswH/AAvxfay/srWeLUT9ca4mrV4uEE9HjLO6mlds39urpkdipbS4G/4rf9TZh5fqczH9LCWvJ7UhoX4Nw4k0B2YUI3rlRSF9rp15ql/YWVrb/Wp2towluCqVABY/ESoHj1wxgZGgiUhEWUTd+VNZsv3cunTwztRk9Xgh47g0Ab5ZZ+Wyd33Nfjx70OukeYF+zFMP9WSn6mx/LZP5qfHh3tnTfMQH93c18fUb/mrB+WyfzSvjw70z8qxy2vmC0m12O7fSUL/WkAklJrGwT4FPxUkKnMTXaXUywyGIEZf4P9N/xLZizY+Lc7PTP0v+V7BQI76tNgLW+T4h/qE1BzmfyPbQ6H/Txk5gz6bvDDtYvNJufMOrxaU07aSmizym3uPXAFxGvLmqXBLoVbjwbN92bDURxVqP7y5f6T+H6WjLKJPo+lG/lhcwzJcxC3CXEVuPWuuTFpQ0tUBU/CvpgU+H7WbANJfTcm1PkP1ZJi3C++KotHqMCX//1pHk1bxV2KsL/Nun+DJ6/wC/4P8AiYxV4xcGskX/ABhj/wCIjCxXRnbCqIQ4qi4ThQmFu2KEztX6YVTSB+mFCA0GSnnzUz/xVbfqkwDmk8kv/Nih0jSV+zymuB0Apsew2xid2UuQZd5U8922r+Wpmey+qC0uIJLzgzTApamJwo+FCobb4RzzB1GWqiBfG3Yo9e5NJfOWm3WhabeXNjJZ2kIuIzYyUNw00qUV9hxqU5kCmVTzCWQYwOKvVxfzeH0sxEiJkerIZ/O2gIC11KYkuZLQ2WmKwEjpD6nMgFgH4vw5lC32U/ycqvjziQG0BKP4/rfwsuWOj/Elum6/osHmqU3r+pfXEl1cxogqgidYhGZH6r+7/Z4/F8eWY9RAiWXfh26LKJoR6sV/M+/vru3Elxc/WEttBQD4w4S5eVhP06P8EYav8uHsuERKRAr1/wCw/hRqjcQP6Lxpp3JrXN3xOupmuk1by9buf99Sf8bZjT5t8OTz+/Oy+NBXIFITvy0ANac9ktEWnsyJUfrzofZmF6gk9If76LrO1pViH9ZlRkVUbioGx7DO58OHUD5PPCcu972Pyx8vyCJotJsJIWjQ1cyK4PAVJ4H4iW+LPlfL7d9o8cv30x6pcP7vDw8PF/Tx/wA19M/krTcuCP2qDfll5X5vHPpdvBIKMgSW4IKUNVqW7EL8Q+L4sR7c9pcxl4v+SOm/6pMx2Rpj/B/sp/rSPzZ5D8p6d5U1HU4LFYLu29MQmO5lmH7yUICwY0751Hsf7U67WdqYdPmlHLhy8fHxYcOL+7xTyf5OEP5rq+1uzcGHTynCPDKP9Ocv4ox/il/SecafKscySxVimjNUkQlWU+II3Ge8HQ4f5sXi8eeV82NajO8vmbzVMzF3XSJg7sSzEssK1JO/7eef9swjHVTjEcIjX+5el0ZvGCUd+U5/f6l/zDx/8nDmuDeX1FIdh8h+rJMVqN8WKoyJtsCX/9eR5NXDFW8VYT+bv/KFz/8AMRB/ycGKvFp2+KL/AIxR/wDERhYr4jhVEI2KouFsKEdA3TFUytnwoTOB+mFUt0aSnnXVDX/ddt+p8A5qeSG/NYn9D6KelZrjbYfq2wDmzPIJ1+SGl2wiu7zUJ/QtDcwlkkNI2jVTKDQ7OWeEf8i8xZyjxizu2RvhZ/5V1KwvtSvdZnMcNpFdXvp+oVBLRySQRlQdyWQE1/ysowwAzSP49TfkkTjiue3ih0Ca8uZIXu7z6haWTPwYqsrR1IXotGmb/KbGER4RA/pIlL94D7l2raTFFpEB4xjWNSvDKZioaYQxigVf5QyxqvFf2cObHeKv6q4p1kv3sZ/N2y07SvLiWEFvHHfyWM91qMyAB3keRKcyOpqz9fs5m4xVDucaW9vBDIemX8TTT0HQ9/LFuf8AiqT/AI2yqXNtHJ5zqdRUHYjtkCoZH5eQfpvUSOiJGo+7+zOq9lh+8yH+jF1HbB9Efe910f8AJ/Sr/RdPv2v7tZLy2iuHEccciK0iBiop8Xw175yPav8AwTdTpdXlwDTRnHBlni45TnDjjjlwcf0cPqdnpvZvFkxRnxyucYy/0wTSw/KeOzkWSLVJZVY7RXNpKwHEHY8JY6Vrmi1f/BS8UGMtMMZ/nY88OL/pZp8jnYOwTjO2Ti/rx/4/BGf8q+uUeJV1ChZmccYL5BR60Ulbk8eNcoH/AAQtPIHiwzGw/i0mT6f4vXpo8XE3fyTMfx/9NI/9Pkq1P8rdcunlibzFJ9WkYEWjpdyRihqB8bvWhFfizb6P/gl9m4qkNKfEiP76I00Mn/Svw/8AYuFn7Az5LHingP8AB6pQ/wBlOTFPMvkW68tWtvdvexXcc8xgAjV0IYLy35e2d/7Me2eDtic4YoZMRwxjOXi8H8fp9Phyl/Nef7R7GnowJGQlxHheaTGt950nP7NmkNf+MskK/wDGmaXtk3qsnv8A96Ha6P8Auoo/8rZfTl1JgKn0oFp/rTUzWhvL6mkbZfkMkxUlPxYqjYWwJf/QkQyatjFW8KsK/NwA+TZQf2riAD5l9vxxV4nchkmVHFHRFVl8CooRihdGcUIhDhVFRNihGwthVMLd+mFCYwS0I3xVLdIk/wCdv1Q/8V2/6nwDmnos/NQO+h6Gsa/vDNOqrtuxqANvh6+GBl0emWvlLTtJ8sXMiR+kVjttMovwiVzQOzD9qR2b7bfs5ga7DGURIj1Yzxx/3Lk6aXqr+cmFj5V0qz0ayiaNqarNNeiM0KpGKVpyqQrs4ZqfaZ2zC1emIAzD+9jHg5/w/wDFf0nIwTiZmP8AD/ChvMXlpm1Cx0aGWRZgsc8Mg2eJ5JeURbb4vSWNAqty+FMli0px5K5+LXif5o9bEzjKBP8AN+n/AHqIuPLST+brcWFxIstrL6cwYfuWit0JkPHceq5k9NmXh/ssli0p4JYeIkfwz/j9X/EsJTAqfVgv5rcI4p2jm9b17KZlRSXWOBXUoeR3FWai/wA/+wyzsvLIjhlf7v0+pdXjEaI/ieMlxXNvbgU9D0JgfK9v/wAYpP8AjbIHmzHJ5zeGrqPcZAqGVeVYS+oas46CTiPkrNnYeykd8h/qf750nbJ2j/nM3OraeamTRbPnT7SerHv40D5vv5PydM2Wv6Xhy/6duF+egRvjh/sv1okeZLBWUppbRAfaWO9ulB+XxGmYw7Jy0QcvH5zw4P8Aewi3DtKA5Q4fdkyKsfm6GM1W3vV36LqVyu1OmQn2NKQ+rF/nabFJsHasf5s/+V00QvnQ1kCT6vEpr6fHUpiR0oTXMY+zkSBxQ0kj/F/gmP8Azv4mf8rx33zD/ktJT1jWhq0NvELnUbj0XLcb+dZlFRSq0VTyzK7K7J/KSkeDTY+Ov8Vw/l5en/VPVPiaNXqxmEQDllw/6tITeczMDaed37mWyQf9JQ/5ozi+05cWpyH+m7zTCsY9yZflQaXWp/8AGCL/AJOHMINpfUTnYfIfqybBYp+LAlFwnFX/0ZEMmreKt4VSDzqivpESekJna5iEURVXVpKngGVvhZOfHn/k4hEuTwrzUix67OinkFVK/AIwG4/EFUbcQdlxKAgoztiqujYVRETYqjInwoR0EnTFCPik6YVS7R5P+ds1M/5MH3DlgHNPRd+aQpomiMGJ5TXBAJFBSvTjt92RPNn0Tf8ALvzBq+paPNp8t3JeXdpLHHZWt07yq8k7j0n5tUp6Xxr8L/Y4/BmFqYmZEAaB+puwnh9XczK3ufObXtpZQumr6xprSpPNJJ6MbW4+JloE4r6bqipVPi4fE3xZjkSzT4eLhhw/T/S4g3V4Y4qso19X84jVE1C1gS8vliWW6vDxMUavzSKqFgAxAVm9J/h/ly2EpGRyH6Y3wsCKHB/EaXQeYPMVjq01vBZr9Vdmt7nUX+L/AEq5l9SZI3B/3UGqeSf7P4cY5JQiZy+qZ5fBHBxGh/CwLz5pscOlXl3biU2cOkQ6ZG8y09Q2krK0iP8AZlVuX2lyegxzjE8YFzlx/wCnRqJiRFdI8LyCozPcVn2hSyf4fgT0m9NYGZZgVoSedRQkN8NPDBTK2BgF7y3UitZEqPbkK5AqmGl+ZLnSLi8EUKTCaVi3MkHYkbUzbdm9rz0gIERLiLianRjKQSapMv8AlYVx+1YRfRIw/wCNTm1HtXPrCP8ApnEPZMe9tPzCUPyNigI6UkDD7mWmTHtYeuP/AGf/AB1h/I45iX+xVj+YdvIOL2Zp/kekD94CnLo+1OIfwT/0zXLsiR/iH+lVYvPulD7VpP8AR6Z/42GWj2qw9Yz/ANj/AMUgdjyHUI+3/MHy+Kc47hP9gD+pjk4+02nPMTHwZ/yZMdQkkE6zeXPNd2tfTub6y9MnY0M00lD/ALHjnE6nIJ5JSHKU5S/2TuccaiB5J1+VbD65qY/4oir/AMjDlYSX1Ax2HyH6smwcvXAlExYq/wD/0pFlit4q6uKsJ/N1mHk2VlNCtxART2fFBeH3UkkkwkkYs7qpZj1JIxVfGcUKynCqvG2KoqJsUI2GTCqNikwoS/SZKeaNSP8Akw/qbIjmnoifzSNdA0E/8W3Hh4n+X4f+ByJZ9GTflDbyaNaT3k9k9w8sMWpwo/7tTGqSKtGIKnmT8APH7WYOpz+HOJI2l6OJuxx4gQObLNK80wR2Osa2YJTdXNbcilGhlnJPF4/t/uua8yvL4cjizxGYwP1S9cf6n0s8kSYgjorXmv6FZ+Wbe2tAyjVLu0RpqqEaGJ4lk4kH4hQPVjxyGHPCWOUB9WP0yUiXEJd6J1y/0d7LRtDhlYTNM17NVCppKr8Gpu1Cf5eXJlyc8uOeESB9IpOPiEz7ikH52X0D6E+mWb87LTLD0wwp/eu4DAjqrKqJ1+L48z4SBFjk4pD54brkmLPtJYr5VgI6+i//ABtiyYP6FwZ4yg/eKQVr0qDUZFCa6f5euNRumhisS0xBkIS4CClRX7Ub92w0tou40CTQJYLu+S6sPUYpDLHLDLVgKkfYXt7YCFIB2KbRavrLwF7bVpxAsZlZpYLWQCMdWNUG304OENR08O5uxbXNUvLe0jvbS6e7JEZuNNsylACWYsoJooViceFfAj0v5ySPUora5j9JntYZKhjJb6e8R+XKPb8MNM4wrqUu/QiE0W/gLHorJcKf+TVPxxpmnEUUFn5Ul00zJPeXd9HcMIuRVIYYmUcmZV+JnbZf5cQkimSfl3dySNPYiOL/AEWGkZiSkzmWXkRIQSXpT4NvhyQYF9LLGxVSRTYZJgvVKYpVkFMCv//TkIyat4UNHFWFfm6f+dMm/wCM8H/E8QgvDZvtL/qL+rFK+M7YqrIcUK6NhVERvihFRvhVFRSAU3xVAaY9fMOo79RD+HLAOapl+Z/F9A8vqzcVaWcMwoaAnc0XY/7HIyZ9HrVlrOhXPlcpod3Fctf3FpbD0QweO0R0Ry/IBl4xh/2eKtlGpnEQNlniviCbJBDLo9la2t3E08rTT3EyujcpJmCUMn2eVJK7fyrlU4AiA7j+hsjOrSrVfL2m3/neHQrOJH0+0tYLe4VQGQoavIN9wOIHJ/8ALwmFZgR/W/0qiX7sp3pOhafr/mxS1tGbCyupZI5ANwtnSNVDfsoJd+KnK8OniDOAH7v+Z/D6x6kzn6Ynq8d88y3t/NrMUZ9QQ2L3Ez7l5RLKxQjf9lIyWr/k8cs0cSIkdLPD/mrqCLFdzyU75luK9C8vUbQ9PQ7hgAR82OEMuiMu9Mt1NRGtR3oMLBM/y9sBJ5kcU2FtIf8AhkwhBeg6r5T0nU7Ex31kl4IQ0kET1+3xNKEeOEhALx5dH1yK3lh+pyRxzoEkR7eVaKCG4jbbpldNto3y9bTWt9MJk4XFxbmysVVSqq0pCN1AofT5Kv8AxkwhXoTfkt5fkAPr3SyEDmyutOVN6BlOS4WHEp2/5KWFpew3tnql3FPA3KMssDjcFSCClCCpIxpbQV3+RKzzPP8Ap24MrkszSRqdya/slcHCkzJ5vQvLfl610iwsbKMLJLawxwNdFFEj8AByYjf4qYQxZaq7dMVdxGKuAwK//9SQZYhvFWjirCfzeP8Azpk3/MRB/wASxQ8NlPxL/qr+rAlehwoVVbFVVGxVXRsKq6SYoVo5CDhVCaXJ/uevj4iP9RwDmnonH5nEHQPL/f4599j3/wAn4fuyJZdGRflDpT61p6acFeOKZ5Ip50YqxTmJHZCpBBC/By/Yb7OYeTFxZRe4+pyIyAx+bKdN8n6Jq6toUTTL5fgup1uJWcESQWLiMRsRQ8VlA5P9rhF9vK5wl4k5geqMfR+P9Mo4eEDvPqZBrfkl5rm6u4dWeGx0iBKsgNZJJaqq7cXRlQoF4P8AyZi6AeiWYj1z9X+lDbmHqEAdkFFaa3HOurJqptNL9YWMEBLIZTyDSTSBT6cnNlb7cfLjy+P4syeE48JIJ4p/77/iWsDinXSLEfzE8tz2PlG91+VUiOrxNFZiNiGFrbv8IdPsrX1OXw/zccysGMwiLN/8U1ZJcReFk5e1PQfLbf7itNHuv/EsIT0ZDdqCTkmtOPy0hB8zSbf8esn/ABNMQpeppGBk2K+tOmBVyqjGpAJ8TilFxKDgVVKCmKVJkxVfbx/HXwxVMlG2BW6YFW4q/wD/1T+uWIbrirROKsJ/N4/86ZL/AMxEH/EsUPDZftj/AFR+rAltDthVUBxQqq2KqyNhVVV8VVFk3xQoaQ8Y127MgJQ+nyCkA036Eg4BzSnX5lq7aFoBUmRnebgood60AXiN+WCTLo9J8neW7/ynZSS28p+G3SK4NeHK7kUlwKV5Rp25cfi/azX6sTjKM4yrf1R/nR/muTgAkDEhW0O0816L5LEXrwvJc3U0Mc8tB60EjCSQ/stG2z/Z5ry+Lg32MEssxMSr91kj/nRyf8SoxjeP8UE/1nXfMlx5dNxa2QgsZ57fULqFkIn9CN43oxBZXkKoSirxbMTT5pY70865cOI/z+L+L/TNk4cX7wcv4lDVdXmOo6VpM1l6NrbPyLxcqCe5SSNUk5Asknx8v2lzIGpM8JJiYyh9WP8Ai9DWIVLyLG/zm1ZL3QJba3i9O106yeA8TzX1GeMmrj4S3wf8NmbgzjJEEbbfS0zgYl89E75c1s/8vN/uM0z5r/xLCEnkyS4bc5NrZD+WQH+JZP8AmFk/4mmEKXpzUFckxUmO+BVaLFUZCMCURTbAlYVxVVgSmKotemKuJwKsJxV//9Y8DZNC/CrROKsI/N8/86XL/wAxEH/EsUPDJD8Q+Q/VgSuU4qvBwqqKcUKqtiqqGwquV98VQ+mvTVro/wCp+o4BzVk/n++ltdN8r3kPFpbeaSePnR1LRuGXlSgYVG9MEmTP9N89X3mHytZtJaxafFbO97qIi5MJk/eRihYlhydlkC/HmDq8hI4IjiN/6VydPGjxHYI+985aBqegaXdT272enW6uPTmKPIZZkHEihCFxSSP0yY25Yc2QGQx0b9Mv6LDHYBkyj/FOnyS3E0l6bLQ/9DRIXqHBjMpl5pTkK8I+Vfg+D7XHMTIIZNXAgbwEr/zfpboEjCfggtIeyu/OFzqV/drF/pM89nbyMtXVI1iiMY/a+Fmb/Z5l4pQlklIG9g1yJEAC81863Us/lnUVkiEBe2M7KVKuGMuyknfoeh/mwaWAuRBtOaRoB4wTma4rPfL5/wBxumfNf+JYQnozTUb2xk0e0tY4FS8hklaeZVoWVvsgt1b/AI1yXVgmX5ZH/nZJP+YWT/iaYQxL05jvkkKZO+Kq8OKUbFgVEdsCWqYqrxjFVXFWicVU2OKv/9c72rk0LsKuJxVg35wH/nTJP+YmD/iWKHhrncfIYEtqcVXht8VVFbChUVsVXh8VXK2KofT2/wBydyf9X+OI5qyP8yG5aF5fNa19c1qDWp8RtgLJl/5KzadNb2o1W5jihtpmMMctKSen8aqAdiVdsxhEeKT5N5kfDA82c6BPp+pPe6zemCWyhF7cJZsFoD6kkaj0+pbgh5ch9pnxxR/eSPu/3KJn0gKEOkWjeX5dZ1G0hmuII7eDS6fCqy3DKWMZFD8TTBWZf2VyvFAjHLv9TPIQZju9KJl0e2isE1ee3d728vhHGitRFt7UbgA7UpESW+3/AJWQnjrDt/FX+yWJBnuk35seW49N8ies7v8ApTV0luZLU0McSclCrGN2AHNFpyzLx4owFAU0SkTzfPb6bcqKlDTLKYsw0IFLHTlOxBWv/BYQpZJcdTk2tkP5aH/nZJP+YWT/AImmIUvTid8mxW98CoiLtgSjYsVRHbAlsYqqocVX8sVWlsCqbE4q/wD/0DsDeuTQ3hVonFDBvzfP/OnOKV/0mDYf6xxV4fMjoVLKVDAFa9xgStBxVeGxVcGxVeHwoXh8VbMqopZjRR1OKrNNVvWkuT8KykcQetADvgCSyT8xyDoHl41rUTb1B7+IxKUu8rQta+a7fTbofWIZC8E0GxRlkSrfC/w/sj/gcpz2IEjm2Y6MgCifLusmW61B53kkt1tria3bq8SRO0yHx/bbn/Nz+LIzuIBHMyCx3O6P07zNqI8tXN1NK31m3ktyLZSRHKCYolRkrwqOAZWpyVuWAjhIgOUuJI3Bl1DJv8eatHb6fPNcyTyNO0C2zEuY5ZklowqpJjCn7Dc0XCRZ4O7hUbepF+dvOkuqPAmpTC4le2McRFBRY5QW+EfD2o1OOTx5BIkfzWMocPxYlJfac0IjPHitSBQA79anqcvJ2prrdThaMyWpi+xzXj/wWBJTu56nJNafflq3/OySf8wsn/E0xCl6dWpyTFsYqiIu2BKNiOKq/bAlcuKqi4q3XFWicVU2O+Kv/9E6ByaG64ULWxVgf5xN/wA6ew/5eYf1nFXji3PwrBdqWtyq8aABk2+F0+j/AIPAlQuLd4HAJDo4rFKv2WXxH8V/ZxVYDiq4EeOKrgw8cVXjlStD9xwoclle3VJTbyfVgaJ8DUYjx2wJRgha3kQ3iPFHUFqAc6UrtX54UMz82eWL++8v2Y2lutMDlrYEUkBNHVXAB5bcl2xLJgFr5iFvrserejyljcsYS/coU+1QHv8Ay5VMcQplE0bVLa+0nTYp0t55btrmymtGrCIvTaXj8W7tyAocZxsD38SxNWiLHWNOTSL20aRkmnks2jqppSCRmepFex2xlG5RP83iWJoHzpkVtqGmXFtpYS7iElveTSygsFYRvAIwd6ftHERPiE/0V4hw0n3mtbC5v7rUbBFSxl07igqlEdbltjxJ+J04s2Y3Z+LJGPDPefF9X85t1EgTY5UwdoXlYJEA7NsArDNgcZDjCYKa2sRge0hJBZHQEjpUtXIsiyC5HXJNadflxt5lf3tpP+JpiFL1JVOSYr+OKq8a4EouLFVcYErlxVeDirZOKrScVWMcCv8A/9I3ByaF1cVbwoY3558r3HmPRv0bbzpbuZo5PUdSwohO1ARjS2w4/kfcx2/K51WE+kCSUt25H2JaU9KbbZLgRxLrf8pbK5gRX1N1j2PpxwxgVApy3r8R7nI0lFxfkhoWxfUrw+yiBf8AmWcPCto2P8l/Kqj45rt/+eir/wARUYaRaJj/ACh8np1S6f53Mo/4iRjS2i4fyx8nxCgs5GH+XcTt+t8aW0W/5eeTltiRpMLv+zzLtv8ASxyXCKY3up2fkbynHQyaHZFvEwqT+IwcKbVp/JVjLK8seoXlu8jFiEdCoJNdlZCAMeFPEll9+Wlo8Mj/AFpJyATS5tIHr8yoTAYpE0il/KuGTcW+nP8AKCSE/wDCOcjSbQE/5QOSSlhAfeO8mQ/8C6kYrsgJ/wApr6MHhY3f/PGe3k/4nxOG0bJbcflxqkIJEF9H48rYSf8AJpjXDa0u0/S4tKhb1Y5/rLfbmlt5YtvABl2GApCnHeWkmoQKk6MwlSqhhX7Q7YKW2faR5Q1rWGDxRehak73MwKqR/kj7T/R8P+VkmDP/AC75M0vRGM0Zae8ZeDzvtsSCQqjZRthAQnnBfDFWigxVUQYqrx4qrA4ErgcVXA4q4nFVpOBVpOKv/9MyDDxyaFwceOKrhIMVXxsPUX55IIKIvWWSJ4RvyFCcsLWEug0+KFQFBoMFMrRSIB2ONItUCjxpjS236f8AlYaW1whr+1jS2qLCKUJrhpCosEfhhpCosCY0tunhQwOtOopgPJQhksxTplbYqiz9sVXC09sUL1tiO2Kqq2pYUIqPfCq1tG052Dy2sUjqaqWRSQR33GKEYF7Yqu9IlSeww0hTK4ErSuKrlGKqq4qqg4FbBxSuDYq4tiq0nFVvLFX/1BZAyxi2AMVXBVw0qrGq8hthAQigTkmC4YVbwq7FW8ULhiq9cKqgJphVepOKFx3/AAwHkkIlVXwypmqBV8MVXcV8MKr1RfDFC+gA6YqtOKuGFVSL7DZIMSoEZBksOKuGKqi4qvxVvAreKuPTFVpxVacUv//V/9n/4gxYSUNDX1BST0ZJTEUAAQEAAAxITGlubwIQAABtbnRyUkdCIFhZWiAHzgACAAkABgAxAABhY3NwTVNGVAAAAABJRUMgc1JHQgAAAAAAAAAAAAAAAAAA9tYAAQAAAADTLUhQICAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABFjcHJ0AAABUAAAADNkZXNjAAABhAAAAGx3dHB0AAAB8AAAABRia3B0AAACBAAAABRyWFlaAAACGAAAABRnWFlaAAACLAAAABRiWFlaAAACQAAAABRkbW5kAAACVAAAAHBkbWRkAAACxAAAAIh2dWVkAAADTAAAAIZ2aWV3AAAD1AAAACRsdW1pAAAD+AAAABRtZWFzAAAEDAAAACR0ZWNoAAAEMAAAAAxyVFJDAAAEPAAACAxnVFJDAAAEPAAACAxiVFJDAAAEPAAACAx0ZXh0AAAAAENvcHlyaWdodCAoYykgMTk5OCBIZXdsZXR0LVBhY2thcmQgQ29tcGFueQAAZGVzYwAAAAAAAAASc1JHQiBJRUM2MTk2Ni0yLjEAAAAAAAAAAAAAABJzUkdCIElFQzYxOTY2LTIuMQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAWFlaIAAAAAAAAPNRAAEAAAABFsxYWVogAAAAAAAAAAAAAAAAAAAAAFhZWiAAAAAAAABvogAAOPUAAAOQWFlaIAAAAAAAAGKZAAC3hQAAGNpYWVogAAAAAAAAJKAAAA+EAAC2z2Rlc2MAAAAAAAAAFklFQyBodHRwOi8vd3d3LmllYy5jaAAAAAAAAAAAAAAAFklFQyBodHRwOi8vd3d3LmllYy5jaAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkZXNjAAAAAAAAAC5JRUMgNjE5NjYtMi4xIERlZmF1bHQgUkdCIGNvbG91ciBzcGFjZSAtIHNSR0IAAAAAAAAAAAAAAC5JRUMgNjE5NjYtMi4xIERlZmF1bHQgUkdCIGNvbG91ciBzcGFjZSAtIHNSR0IAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZGVzYwAAAAAAAAAsUmVmZXJlbmNlIFZpZXdpbmcgQ29uZGl0aW9uIGluIElFQzYxOTY2LTIuMQAAAAAAAAAAAAAALFJlZmVyZW5jZSBWaWV3aW5nIENvbmRpdGlvbiBpbiBJRUM2MTk2Ni0yLjEAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAHZpZXcAAAAAABOk/gAUXy4AEM8UAAPtzAAEEwsAA1yeAAAAAVhZWiAAAAAAAEwJVgBQAAAAVx/nbWVhcwAAAAAAAAABAAAAAAAAAAAAAAAAAAAAAAAAAo8AAAACc2lnIAAAAABDUlQgY3VydgAAAAAAAAQAAAAABQAKAA8AFAAZAB4AIwAoAC0AMgA3ADsAQABFAEoATwBUAFkAXgBjAGgAbQByAHcAfACBAIYAiwCQAJUAmgCfAKQAqQCuALIAtwC8AMEAxgDLANAA1QDbAOAA5QDrAPAA9gD7AQEBBwENARMBGQEfASUBKwEyATgBPgFFAUwBUgFZAWABZwFuAXUBfAGDAYsBkgGaAaEBqQGxAbkBwQHJAdEB2QHhAekB8gH6AgMCDAIUAh0CJgIvAjgCQQJLAlQCXQJnAnECegKEAo4CmAKiAqwCtgLBAssC1QLgAusC9QMAAwsDFgMhAy0DOANDA08DWgNmA3IDfgOKA5YDogOuA7oDxwPTA+AD7AP5BAYEEwQgBC0EOwRIBFUEYwRxBH4EjASaBKgEtgTEBNME4QTwBP4FDQUcBSsFOgVJBVgFZwV3BYYFlgWmBbUFxQXVBeUF9gYGBhYGJwY3BkgGWQZqBnsGjAadBq8GwAbRBuMG9QcHBxkHKwc9B08HYQd0B4YHmQesB78H0gflB/gICwgfCDIIRghaCG4IggiWCKoIvgjSCOcI+wkQCSUJOglPCWQJeQmPCaQJugnPCeUJ+woRCicKPQpUCmoKgQqYCq4KxQrcCvMLCwsiCzkLUQtpC4ALmAuwC8gL4Qv5DBIMKgxDDFwMdQyODKcMwAzZDPMNDQ0mDUANWg10DY4NqQ3DDd4N+A4TDi4OSQ5kDn8Omw62DtIO7g8JDyUPQQ9eD3oPlg+zD88P7BAJECYQQxBhEH4QmxC5ENcQ9RETETERTxFtEYwRqhHJEegSBxImEkUSZBKEEqMSwxLjEwMTIxNDE2MTgxOkE8UT5RQGFCcUSRRqFIsUrRTOFPAVEhU0FVYVeBWbFb0V4BYDFiYWSRZsFo8WshbWFvoXHRdBF2UXiReuF9IX9xgbGEAYZRiKGK8Y1Rj6GSAZRRlrGZEZtxndGgQaKhpRGncanhrFGuwbFBs7G2MbihuyG9ocAhwqHFIcexyjHMwc9R0eHUcdcB2ZHcMd7B4WHkAeah6UHr4e6R8THz4faR+UH78f6iAVIEEgbCCYIMQg8CEcIUghdSGhIc4h+yInIlUigiKvIt0jCiM4I2YjlCPCI/AkHyRNJHwkqyTaJQklOCVoJZclxyX3JicmVyaHJrcm6CcYJ0kneierJ9woDSg/KHEooijUKQYpOClrKZ0p0CoCKjUqaCqbKs8rAis2K2krnSvRLAUsOSxuLKIs1y0MLUEtdi2rLeEuFi5MLoIuty7uLyQvWi+RL8cv/jA1MGwwpDDbMRIxSjGCMbox8jIqMmMymzLUMw0zRjN/M7gz8TQrNGU0njTYNRM1TTWHNcI1/TY3NnI2rjbpNyQ3YDecN9c4FDhQOIw4yDkFOUI5fzm8Ofk6Njp0OrI67zstO2s7qjvoPCc8ZTykPOM9Ij1hPaE94D4gPmA+oD7gPyE/YT+iP+JAI0BkQKZA50EpQWpBrEHuQjBCckK1QvdDOkN9Q8BEA0RHRIpEzkUSRVVFmkXeRiJGZ0arRvBHNUd7R8BIBUhLSJFI10kdSWNJqUnwSjdKfUrESwxLU0uaS+JMKkxyTLpNAk1KTZNN3E4lTm5Ot08AT0lPk0/dUCdQcVC7UQZRUFGbUeZSMVJ8UsdTE1NfU6pT9lRCVI9U21UoVXVVwlYPVlxWqVb3V0RXklfgWC9YfVjLWRpZaVm4WgdaVlqmWvVbRVuVW+VcNVyGXNZdJ114XcleGl5sXr1fD19hX7NgBWBXYKpg/GFPYaJh9WJJYpxi8GNDY5dj62RAZJRk6WU9ZZJl52Y9ZpJm6Gc9Z5Nn6Wg/aJZo7GlDaZpp8WpIap9q92tPa6dr/2xXbK9tCG1gbbluEm5rbsRvHm94b9FwK3CGcOBxOnGVcfByS3KmcwFzXXO4dBR0cHTMdSh1hXXhdj52m3b4d1Z3s3gReG54zHkqeYl553pGeqV7BHtje8J8IXyBfOF9QX2hfgF+Yn7CfyN/hH/lgEeAqIEKgWuBzYIwgpKC9INXg7qEHYSAhOOFR4Wrhg6GcobXhzuHn4gEiGmIzokziZmJ/opkisqLMIuWi/yMY4zKjTGNmI3/jmaOzo82j56QBpBukNaRP5GokhGSepLjk02TtpQglIqU9JVflcmWNJaflwqXdZfgmEyYuJkkmZCZ/JpomtWbQpuvnByciZz3nWSd0p5Anq6fHZ+Ln/qgaaDYoUehtqImopajBqN2o+akVqTHpTilqaYapoum/adup+CoUqjEqTepqaocqo+rAqt1q+msXKzQrUStuK4trqGvFq+LsACwdbDqsWCx1rJLssKzOLOutCW0nLUTtYq2AbZ5tvC3aLfguFm40blKucK6O7q1uy67p7whvJu9Fb2Pvgq+hL7/v3q/9cBwwOzBZ8Hjwl/C28NYw9TEUcTOxUvFyMZGxsPHQce/yD3IvMk6ybnKOMq3yzbLtsw1zLXNNc21zjbOts83z7jQOdC60TzRvtI/0sHTRNPG1EnUy9VO1dHWVdbY11zX4Nhk2OjZbNnx2nba+9uA3AXcit0Q3ZbeHN6i3ynfr+A24L3hROHM4lPi2+Nj4+vkc+T85YTmDeaW5x/nqegy6LzpRunQ6lvq5etw6/vshu0R7ZzuKO6070DvzPBY8OXxcvH/8ozzGfOn9DT0wvVQ9d72bfb794r4Gfio+Tj5x/pX+uf7d/wH/Jj9Kf26/kv+3P9t////7QBmUGhvdG9zaG9wIDMuMAA4QklNBAQAAAAAAEkcAVoAAxslRxwCAAACAAQcAjcACDIwMjYwMTIyHAI8AAsxMTU0MDQtMDUwMBwCPgAIMjAyNjAxMjIcAj8ACzExNTQwNS0wNTAwAP/hl5NodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvADw/eHBhY2tldCBiZWdpbj0i77u/IiBpZD0iVzVNME1wQ2VoaUh6cmVTek5UY3prYzlkIj8+Cjx4OnhtcG1ldGEgeG1sbnM6eD0iYWRvYmU6bnM6bWV0YS8iIHg6eG1wdGs9IkFkb2JlIFhNUCBDb3JlIDcuMC1jMDAwIDEuMDAwMDAwLCAwMDAwLzAwLzAwLTAwOjAwOjAwICAgICAgICAiPgogPHJkZjpSREYgeG1sbnM6cmRmPSJodHRwOi8vd3d3LnczLm9yZy8xOTk5LzAyLzIyLXJkZi1zeW50YXgtbnMjIj4KICA8cmRmOkRlc2NyaXB0aW9uIHJkZjphYm91dD0iIgogICAgeG1sbnM6eG1wPSJodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvIgogICAgeG1sbnM6YXV4PSJodHRwOi8vbnMuYWRvYmUuY29tL2V4aWYvMS4wL2F1eC8iCiAgICB4bWxuczpleGlmRVg9Imh0dHA6Ly9jaXBhLmpwL2V4aWYvMS4wLyIKICAgIHhtbG5zOnBob3Rvc2hvcD0iaHR0cDovL25zLmFkb2JlLmNvbS9waG90b3Nob3AvMS4wLyIKICAgIHhtbG5zOnhtcE1NPSJodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvbW0vIgogICAgeG1sbnM6c3RFdnQ9Imh0dHA6Ly9ucy5hZG9iZS5jb20veGFwLzEuMC9zVHlwZS9SZXNvdXJjZUV2ZW50IyIKICAgIHhtbG5zOnN0UmVmPSJodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvc1R5cGUvUmVzb3VyY2VSZWYjIgogICAgeG1sbnM6ZGM9Imh0dHA6Ly9wdXJsLm9yZy9kYy9lbGVtZW50cy8xLjEvIgogICAgeG1sbnM6eG1wRE09Imh0dHA6Ly9ucy5hZG9iZS5jb20veG1wLzEuMC9EeW5hbWljTWVkaWEvIgogICAgeG1sbnM6Y3JzPSJodHRwOi8vbnMuYWRvYmUuY29tL2NhbWVyYS1yYXctc2V0dGluZ3MvMS4wLyIKICAgeG1wOk1vZGlmeURhdGU9IjIwMjYtMDItMTJUMDQ6MTE6MTArMDY6MDAiCiAgIHhtcDpDcmVhdGVEYXRlPSIyMDI2LTAxLTIyVDExOjU0OjA1LjEzMS0wNTowMCIKICAgeG1wOk1ldGFkYXRhRGF0ZT0iMjAyNi0wMi0xMlQwNDoxMToxMCswNjowMCIKICAgeG1wOkNyZWF0b3JUb29sPSJBZG9iZSBQaG90b3Nob3AgTGlnaHRyb29tIENsYXNzaWMgMTUuMS4xIChNYWNpbnRvc2gpIgogICB4bXA6UmF0aW5nPSIzIgogICBhdXg6U2VyaWFsTnVtYmVyPSIxNTIyMDI0MDAzMDEiCiAgIGF1eDpMZW5zSW5mbz0iOTAvMSA5MC8xIDAvMCAwLzAiCiAgIGF1eDpMZW5zPSJUUy1FOTBtbSBmLzIuOCIKICAgYXV4OkxlbnNJRD0iMTI3IgogICBhdXg6TGVuc1NlcmlhbE51bWJlcj0iMDAwMDAwMDAwMCIKICAgYXV4OkltYWdlTnVtYmVyPSIwIgogICBhdXg6Rmxhc2hDb21wZW5zYXRpb249IjAvMSIKICAgYXV4OkZpcm13YXJlPSIxLjIuMCIKICAgYXV4OklzTWVyZ2VkSERSPSJUcnVlIgogICBhdXg6TGF0ZXJhbENocm9tYXRpY0FiZXJyYXRpb25Db3JyZWN0aW9uQWxyZWFkeUFwcGxpZWQ9IlRydWUiCiAgIGV4aWZFWDpMZW5zTW9kZWw9IlRTLUU5MG1tIGYvMi44IgogICBwaG90b3Nob3A6RGF0ZUNyZWF0ZWQ9IjIwMjYtMDEtMjJUMTE6NTQ6MDQuMzktMDU6MDAiCiAgIHhtcE1NOkRvY3VtZW50SUQ9InhtcC5kaWQ6NjQxNzg4YjItNDg2Yi00ZDkxLWFjMWEtNDI4NTE0ZDM3YjE5IgogICB4bXBNTTpQcmVzZXJ2ZWRGaWxlTmFtZT0iSFNodF8wMTcwLkNSMyIKICAgeG1wTU06T3JpZ2luYWxEb2N1bWVudElEPSIzOEU2MEY4M0EyRDYyQkRDQzRCQTdEMTZEMkM1Q0QxOSIKICAgeG1wTU06SW5zdGFuY2VJRD0ieG1wLmlpZDo2NDE3ODhiMi00ODZiLTRkOTEtYWMxYS00Mjg1MTRkMzdiMTkiCiAgIGRjOmZvcm1hdD0iaW1hZ2UvanBlZyIKICAgeG1wRE06cGljaz0iMCIKICAgY3JzOlJhd0ZpbGVOYW1lPSJIU2h0XzAxNzAtSERSLmpwZyIKICAgY3JzOlZlcnNpb249IjE4LjEiCiAgIGNyczpDb21wYXRpYmxlVmVyc2lvbj0iMjY4NDM1NDU2IgogICBjcnM6UHJvY2Vzc1ZlcnNpb249IjE1LjQiCiAgIGNyczpXaGl0ZUJhbGFuY2U9IkFzIFNob3QiCiAgIGNyczpJbmNyZW1lbnRhbFRlbXBlcmF0dXJlPSIwIgogICBjcnM6SW5jcmVtZW50YWxUaW50PSIwIgogICBjcnM6RXhwb3N1cmUyMDEyPSIwLjAwIgogICBjcnM6Q29udHJhc3QyMDEyPSIwIgogICBjcnM6SGlnaGxpZ2h0czIwMTI9IjAiCiAgIGNyczpTaGFkb3dzMjAxMj0iMCIKICAgY3JzOldoaXRlczIwMTI9IjAiCiAgIGNyczpCbGFja3MyMDEyPSIwIgogICBjcnM6VGV4dHVyZT0iMCIKICAgY3JzOkNsYXJpdHkyMDEyPSIwIgogICBjcnM6RGVoYXplPSIwIgogICBjcnM6VmlicmFuY2U9IjAiCiAgIGNyczpTYXR1cmF0aW9uPSIwIgogICBjcnM6UGFyYW1ldHJpY1NoYWRvd3M9IjAiCiAgIGNyczpQYXJhbWV0cmljRGFya3M9IjAiCiAgIGNyczpQYXJhbWV0cmljTGlnaHRzPSIwIgogICBjcnM6UGFyYW1ldHJpY0hpZ2hsaWdodHM9IjAiCiAgIGNyczpQYXJhbWV0cmljU2hhZG93U3BsaXQ9IjI1IgogICBjcnM6UGFyYW1ldHJpY01pZHRvbmVTcGxpdD0iNTAiCiAgIGNyczpQYXJhbWV0cmljSGlnaGxpZ2h0U3BsaXQ9Ijc1IgogICBjcnM6U2hhcnBuZXNzPSIwIgogICBjcnM6THVtaW5hbmNlU21vb3RoaW5nPSIwIgogICBjcnM6Q29sb3JOb2lzZVJlZHVjdGlvbj0iMCIKICAgY3JzOkh1ZUFkanVzdG1lbnRSZWQ9IjAiCiAgIGNyczpIdWVBZGp1c3RtZW50T3JhbmdlPSIwIgogICBjcnM6SHVlQWRqdXN0bWVudFllbGxvdz0iMCIKICAgY3JzOkh1ZUFkanVzdG1lbnRHcmVlbj0iMCIKICAgY3JzOkh1ZUFkanVzdG1lbnRBcXVhPSIwIgogICBjcnM6SHVlQWRqdXN0bWVudEJsdWU9IjAiCiAgIGNyczpIdWVBZGp1c3RtZW50UHVycGxlPSIwIgogICBjcnM6SHVlQWRqdXN0bWVudE1hZ2VudGE9IjAiCiAgIGNyczpTYXR1cmF0aW9uQWRqdXN0bWVudFJlZD0iMCIKICAgY3JzOlNhdHVyYXRpb25BZGp1c3RtZW50T3JhbmdlPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRZZWxsb3c9IjAiCiAgIGNyczpTYXR1cmF0aW9uQWRqdXN0bWVudEdyZWVuPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRBcXVhPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRCbHVlPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRQdXJwbGU9IjAiCiAgIGNyczpTYXR1cmF0aW9uQWRqdXN0bWVudE1hZ2VudGE9IjAiCiAgIGNyczpMdW1pbmFuY2VBZGp1c3RtZW50UmVkPSIwIgogICBjcnM6THVtaW5hbmNlQWRqdXN0bWVudE9yYW5nZT0iMCIKICAgY3JzOkx1bWluYW5jZUFkanVzdG1lbnRZZWxsb3c9IjAiCiAgIGNyczpMdW1pbmFuY2VBZGp1c3RtZW50R3JlZW49IjAiCiAgIGNyczpMdW1pbmFuY2VBZGp1c3RtZW50QXF1YT0iMCIKICAgY3JzOkx1bWluYW5jZUFkanVzdG1lbnRCbHVlPSIwIgogICBjcnM6THVtaW5hbmNlQWRqdXN0bWVudFB1cnBsZT0iMCIKICAgY3JzOkx1bWluYW5jZUFkanVzdG1lbnRNYWdlbnRhPSIwIgogICBjcnM6U3BsaXRUb25pbmdTaGFkb3dIdWU9IjAiCiAgIGNyczpTcGxpdFRvbmluZ1NoYWRvd1NhdHVyYXRpb249IjAiCiAgIGNyczpTcGxpdFRvbmluZ0hpZ2hsaWdodEh1ZT0iMCIKICAgY3JzOlNwbGl0VG9uaW5nSGlnaGxpZ2h0U2F0dXJhdGlvbj0iMCIKICAgY3JzOlNwbGl0VG9uaW5nQmFsYW5jZT0iMCIKICAgY3JzOkNvbG9yR3JhZGVNaWR0b25lSHVlPSIwIgogICBjcnM6Q29sb3JHcmFkZU1pZHRvbmVTYXQ9IjAiCiAgIGNyczpDb2xvckdyYWRlU2hhZG93THVtPSIwIgogICBjcnM6Q29sb3JHcmFkZU1pZHRvbmVMdW09IjAiCiAgIGNyczpDb2xvckdyYWRlSGlnaGxpZ2h0THVtPSIwIgogICBjcnM6Q29sb3JHcmFkZUJsZW5kaW5nPSI1MCIKICAgY3JzOkNvbG9yR3JhZGVHbG9iYWxIdWU9IjAiCiAgIGNyczpDb2xvckdyYWRlR2xvYmFsU2F0PSIwIgogICBjcnM6Q29sb3JHcmFkZUdsb2JhbEx1bT0iMCIKICAgY3JzOkF1dG9MYXRlcmFsQ0E9IjAiCiAgIGNyczpMZW5zUHJvZmlsZUVuYWJsZT0iMCIKICAgY3JzOkxlbnNNYW51YWxEaXN0b3J0aW9uQW1vdW50PSIwIgogICBjcnM6VmlnbmV0dGVBbW91bnQ9IjAiCiAgIGNyczpEZWZyaW5nZVB1cnBsZUFtb3VudD0iMCIKICAgY3JzOkRlZnJpbmdlUHVycGxlSHVlTG89IjMwIgogICBjcnM6RGVmcmluZ2VQdXJwbGVIdWVIaT0iNzAiCiAgIGNyczpEZWZyaW5nZUdyZWVuQW1vdW50PSIwIgogICBjcnM6RGVmcmluZ2VHcmVlbkh1ZUxvPSI0MCIKICAgY3JzOkRlZnJpbmdlR3JlZW5IdWVIaT0iNjAiCiAgIGNyczpQZXJzcGVjdGl2ZVVwcmlnaHQ9IjAiCiAgIGNyczpQZXJzcGVjdGl2ZVZlcnRpY2FsPSIwIgogICBjcnM6UGVyc3BlY3RpdmVIb3Jpem9udGFsPSIwIgogICBjcnM6UGVyc3BlY3RpdmVSb3RhdGU9IjAuMCIKICAgY3JzOlBlcnNwZWN0aXZlQXNwZWN0PSIwIgogICBjcnM6UGVyc3BlY3RpdmVTY2FsZT0iMTAwIgogICBjcnM6UGVyc3BlY3RpdmVYPSIwLjAwIgogICBjcnM6UGVyc3BlY3RpdmVZPSIwLjAwIgogICBjcnM6R3JhaW5BbW91bnQ9IjAiCiAgIGNyczpQb3N0Q3JvcFZpZ25ldHRlQW1vdW50PSIwIgogICBjcnM6U2hhZG93VGludD0iMCIKICAgY3JzOlJlZEh1ZT0iMCIKICAgY3JzOlJlZFNhdHVyYXRpb249IjAiCiAgIGNyczpHcmVlbkh1ZT0iMCIKICAgY3JzOkdyZWVuU2F0dXJhdGlvbj0iMCIKICAgY3JzOkJsdWVIdWU9IjAiCiAgIGNyczpCbHVlU2F0dXJhdGlvbj0iMCIKICAgY3JzOkhEUkVkaXRNb2RlPSIwIgogICBjcnM6Q29udmVydFRvR3JheXNjYWxlPSJGYWxzZSIKICAgY3JzOk92ZXJyaWRlTG9va1ZpZ25ldHRlPSJGYWxzZSIKICAgY3JzOlRvbmVDdXJ2ZU5hbWUyMDEyPSJMaW5lYXIiCiAgIGNyczpDYW1lcmFQcm9maWxlPSJFbWJlZGRlZCIKICAgY3JzOkNhbWVyYVByb2ZpbGVEaWdlc3Q9IjU0NjUwQTM0MUI1QjVDQ0FFODQ0MkQwQjQzQTkyQkNFIgogICBjcnM6SGFzU2V0dGluZ3M9IlRydWUiCiAgIGNyczpDcm9wVG9wPSIwIgogICBjcnM6Q3JvcExlZnQ9IjAiCiAgIGNyczpDcm9wQm90dG9tPSIxIgogICBjcnM6Q3JvcFJpZ2h0PSIxIgogICBjcnM6Q3JvcEFuZ2xlPSIwIgogICBjcnM6Q3JvcENvbnN0cmFpblRvV2FycD0iMCIKICAgY3JzOkNyb3BDb25zdHJhaW5Ub1VuaXRTcXVhcmU9IjEiCiAgIGNyczpIYXNDcm9wPSJGYWxzZSIKICAgY3JzOkFscmVhZHlBcHBsaWVkPSJUcnVlIj4KICAgPHhtcE1NOkhpc3Rvcnk+CiAgICA8cmRmOlNlcT4KICAgICA8cmRmOmxpCiAgICAgIHN0RXZ0OmFjdGlvbj0iZGVyaXZlZCIKICAgICAgc3RFdnQ6cGFyYW1ldGVycz0ic2F2ZWQgdG8gbmV3IGxvY2F0aW9uIi8+CiAgICAgPHJkZjpsaQogICAgICBzdEV2dDphY3Rpb249InNhdmVkIgogICAgICBzdEV2dDppbnN0YW5jZUlEPSJ4bXAuaWlkOmY2NjczNjY2LWFhZDktNGFlNy04ZGNlLWYwMmUwODBiODNjMiIKICAgICAgc3RFdnQ6d2hlbj0iMjAyNi0wMS0zMVQwNDoxODowMSswNjowMCIKICAgICAgc3RFdnQ6c29mdHdhcmVBZ2VudD0iQWRvYmUgUGhvdG9zaG9wIExpZ2h0cm9vbSBDbGFzc2ljIDE1LjEuMSAoTWFjaW50b3NoKSIKICAgICAgc3RFdnQ6Y2hhbmdlZD0iLyIvPgogICAgIDxyZGY6bGkKICAgICAgc3RFdnQ6YWN0aW9uPSJkZXJpdmVkIgogICAgICBzdEV2dDpwYXJhbWV0ZXJzPSJjb252ZXJ0ZWQgZnJvbSBpbWFnZS9kbmcgdG8gaW1hZ2UvanBlZywgc2F2ZWQgdG8gbmV3IGxvY2F0aW9uIi8+CiAgICAgPHJkZjpsaQogICAgICBzdEV2dDphY3Rpb249InNhdmVkIgogICAgICBzdEV2dDppbnN0YW5jZUlEPSJ4bXAuaWlkOjIyOGY2NGFmLTJkYjgtNGFjZC1iNWVhLTQzOGIxZTI2MGVmZCIKICAgICAgc3RFdnQ6d2hlbj0iMjAyNi0wMi0wN1QwOTowMzo0NiswNjowMCIKICAgICAgc3RFdnQ6c29mdHdhcmVBZ2VudD0iQWRvYmUgUGhvdG9zaG9wIExpZ2h0cm9vbSBDbGFzc2ljIDE1LjEuMSAoTWFjaW50b3NoKSIKICAgICAgc3RFdnQ6Y2hhbmdlZD0iLyIvPgogICAgIDxyZGY6bGkKICAgICAgc3RFdnQ6YWN0aW9uPSJkZXJpdmVkIgogICAgICBzdEV2dDpwYXJhbWV0ZXJzPSJzYXZlZCB0byBuZXcgbG9jYXRpb24iLz4KICAgICA8cmRmOmxpCiAgICAgIHN0RXZ0OmFjdGlvbj0ic2F2ZWQiCiAgICAgIHN0RXZ0Omluc3RhbmNlSUQ9InhtcC5paWQ6NjQxNzg4YjItNDg2Yi00ZDkxLWFjMWEtNDI4NTE0ZDM3YjE5IgogICAgICBzdEV2dDp3aGVuPSIyMDI2LTAyLTEyVDA0OjExOjEwKzA2OjAwIgogICAgICBzdEV2dDpzb2Z0d2FyZUFnZW50PSJBZG9iZSBQaG90b3Nob3AgTGlnaHRyb29tIENsYXNzaWMgMTUuMS4xIChNYWNpbnRvc2gpIgogICAgICBzdEV2dDpjaGFuZ2VkPSIvIi8+CiAgICA8L3JkZjpTZXE+CiAgIDwveG1wTU06SGlzdG9yeT4KICAgPHhtcE1NOkRlcml2ZWRGcm9tCiAgICBzdFJlZjppbnN0YW5jZUlEPSJ4bXAuaWlkOjIyOGY2NGFmLTJkYjgtNGFjZC1iNWVhLTQzOGIxZTI2MGVmZCIKICAgIHN0UmVmOmRvY3VtZW50SUQ9InhtcC5kaWQ6MjI4ZjY0YWYtMmRiOC00YWNkLWI1ZWEtNDM4YjFlMjYwZWZkIgogICAgc3RSZWY6b3JpZ2luYWxEb2N1bWVudElEPSIzOEU2MEY4M0EyRDYyQkRDQzRCQTdEMTZEMkM1Q0QxOSIvPgogICA8Y3JzOlRvbmVDdXJ2ZVBWMjAxMj4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+MCwgMDwvcmRmOmxpPgogICAgIDxyZGY6bGk+MjU1LCAyNTU8L3JkZjpsaT4KICAgIDwvcmRmOlNlcT4KICAgPC9jcnM6VG9uZUN1cnZlUFYyMDEyPgogICA8Y3JzOlRvbmVDdXJ2ZVBWMjAxMlJlZD4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+MCwgMDwvcmRmOmxpPgogICAgIDxyZGY6bGk+MjU1LCAyNTU8L3JkZjpsaT4KICAgIDwvcmRmOlNlcT4KICAgPC9jcnM6VG9uZUN1cnZlUFYyMDEyUmVkPgogICA8Y3JzOlRvbmVDdXJ2ZVBWMjAxMkdyZWVuPgogICAgPHJkZjpTZXE+CiAgICAgPHJkZjpsaT4wLCAwPC9yZGY6bGk+CiAgICAgPHJkZjpsaT4yNTUsIDI1NTwvcmRmOmxpPgogICAgPC9yZGY6U2VxPgogICA8L2NyczpUb25lQ3VydmVQVjIwMTJHcmVlbj4KICAgPGNyczpUb25lQ3VydmVQVjIwMTJCbHVlPgogICAgPHJkZjpTZXE+CiAgICAgPHJkZjpsaT4wLCAwPC9yZGY6bGk+CiAgICAgPHJkZjpsaT4yNTUsIDI1NTwvcmRmOmxpPgogICAgPC9yZGY6U2VxPgogICA8L2NyczpUb25lQ3VydmVQVjIwMTJCbHVlPgogICA8Y3JzOlBvaW50Q29sb3JzPgogICAgPHJkZjpTZXE+CiAgICAgPHJkZjpsaT4tMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDA8L3JkZjpsaT4KICAgIDwvcmRmOlNlcT4KICAgPC9jcnM6UG9pbnRDb2xvcnM+CiAgIDxjcnM6Q29sb3JWYXJpYW5jZT4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+LTUwLjAwMDAwMDwvcmRmOmxpPgogICAgPC9yZGY6U2VxPgogICA8L2NyczpDb2xvclZhcmlhbmNlPgogICA8Y3JzOlJldG91Y2hBcmVhcz4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+CiAgICAgIDxyZGY6RGVzY3JpcHRpb24KICAgICAgIGNyczpTcG90VHlwZT0iY2xvbmUiCiAgICAgICBjcnM6U291cmNlU3RhdGU9InNvdXJjZUF1dG9Db21wdXRlZCIKICAgICAgIGNyczpNZXRob2Q9ImdhdXNzaWFuIgogICAgICAgY3JzOkhlYWxWZXJzaW9uPSIyIgogICAgICAgY3JzOlNvdXJjZVg9IjAuODAzMjQzIgogICAgICAgY3JzOk9mZnNldFk9IjAuNDEwODI0IgogICAgICAgY3JzOk9wYWNpdHk9IjEiCiAgICAgICBjcnM6RmVhdGhlcj0iMCIKICAgICAgIGNyczpTZWVkPSIyIj4KICAgICAgPGNyczpNYXNrcz4KICAgICAgIDxyZGY6U2VxPgogICAgICAgIDxyZGY6bGk+CiAgICAgICAgIDxyZGY6RGVzY3JpcHRpb24KICAgICAgICAgIGNyczpXaGF0PSJNYXNrL1BhaW50IgogICAgICAgICAgY3JzOk1hc2tBY3RpdmU9InRydWUiCiAgICAgICAgICBjcnM6TWFza0JsZW5kTW9kZT0iMCIKICAgICAgICAgIGNyczpNYXNrSW52ZXJ0ZWQ9ImZhbHNlIgogICAgICAgICAgY3JzOk1hc2tTeW5jSUQ9IkY2NURENTI0NTE1MzRDM0NBNjk1OTRCMjMxMjFGMzk4IgogICAgICAgICAgY3JzOk1hc2tWYWx1ZT0iMSIKICAgICAgICAgIGNyczpSYWRpdXM9IjAuMDAxODU1IgogICAgICAgICAgY3JzOkZsb3c9IjEiCiAgICAgICAgICBjcnM6Q2VudGVyV2VpZ2h0PSIxIj4KICAgICAgICAgPGNyczpEYWJzPgogICAgICAgICAgPHJkZjpTZXE+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA4MDA5IDAuNDEwODI0PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTk2IDAuNDExMzgwPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTg0IDAuNDExOTM1PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTcyIDAuNDEyNDkxPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTE1IDAuNDEzMDQxPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODgxIDAuNDEzNTk0PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODYzIDAuNDE0MTUwPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODU4IDAuNDE0NzA2PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODU4IDAuNDE1MjYyPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODU4IDAuNDE1ODE4PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODgwIDAuNDE2MzczPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA4MDI0IDAuNDE2ODg2PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA4MzgxIDAuNDE3MDM4PC</t>
+          <t>["photos/WO#30583_20260619_1715303358.jpg"]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-06-19 15:36:57</t>
+          <t>2026-06-19 17:15:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -531,54 +531,160 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>30583</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sycamore Manor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A-1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Antonio Smith</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-06-19 17:17:14</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jonathan Morton</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>30583</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Sycamore Manor</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>A-1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Kitchen</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>tech_notes</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Antonio Smith</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-06-19 17:17:14</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jonathan Morton</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>30583</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sycamore Manor</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A-1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>time_log</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>[{"start_date": "2026-06-19", "start_time": "10:36", "end_date": "", "end_time": "11:36"}]</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[{"start_date": "2026-06-19", "start_time": "12:15", "end_date": "2026-06-19", "end_time": "12:16"}]</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Antonio Smith</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2026-06-19 15:36:57</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-06-19 17:17:14</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Jonathan Morton</t>
         </is>
@@ -595,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -705,6 +811,116 @@
         </is>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>Jonathan Morton</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>30583</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sycamore Manor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A-1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>photos</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>["data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEA8ADwAAD/4TCmRXhpZgAASUkqAAgAAAAIAA8BAgAGAAAAbgAAABABAgAPAAAAdAAAABoBBQABAAAAhAAAABsBBQABAAAAjAAAACgBAwABAAAAAgAAADEBAgA1AAAAlAAAADIBAgAUAAAAygAAAGmHBAABAAAA3gAAAEIDAABDYW5vbgBDYW5vbiBFT1MgUjVtMgAA8AAAAAEAAADwAAAAAQAAAEFkb2JlIFBob3Rvc2hvcCBMaWdodHJvb20gQ2xhc3NpYyAxNS4xLjEgKE1hY2ludG9zaCkAADIwMjY6MDI6MTIgMDQ6MTE6MTAAIQCaggUAAQAAAHACAACdggUAAQAAAHgCAAAiiAMAAQAAAAEAAAAniAMAAQAAAKAAAAAwiAMAAQAAAAIAAAAyiAQAAQAAAKAAAAAAkAcABAAAADAyMzEDkAIAFAAAAIACAAAEkAIAFAAAAJQCAAAQkAIABwAAAKgCAAARkAIABwAAALACAAASkAIABwAAALgCAAABkgoAAQAAAMACAAACkgUAAQAAAMgCAAAEkgoAAQAAANACAAAFkgUAAQAAANgCAAAHkgMAAQAAAAUAAAAJkgMAAQAAAAAAAAAKkgUAAQAAAOACAACRkgIABAAAADEzMQCSkgIABAAAADEzMQABoAMAAQAAAAEAAAAOogUAAQAAAOgCAAAPogUAAQAAAPACAAAQogMAAQAAAAIAAAABpAMAAQAAAAAAAAACpAMAAQAAAAEAAAADpAMAAQAAAAEAAAAGpAMAAQAAAAAAAAAxpAIADQAAAPgCAAAypAUABAAAAAYDAAA0pAIADwAAACYDAAA1pAIACwAAADYDAAAAAAAAAQAAADwAAAAFAAAAAQAAADIwMjY6MDE6MjIgMTE6NTQ6MDUAMjAyNjowMToyMiAxMTo1NDowNQArMDY6MDAAAC0wNTowMAAALTA1OjAwAADLIVoAQEIPABDcRgBAQg8AAAAAAAEAAAADAAAAAQAAAFoAAAABAAAAAAB9AIsFAADAX1MAswMAADE1MjIwMjQwMDMwMQAAWgAAAAEAAABaAAAAAQAAAAAAAAAAAAAAAAAAAAAAAABUUy1FOTBtbSBmLzIuOAAAMDAwMDAwMDAwMAAABgADAQMAAQAAAAYAAAAaAQUAAQAAAJADAAAbAQUAAQAAAJgDAAAoAQMAAQAAAAIAAAABAgQAAQAAAKADAAACAgQAAQAAAP4sAAAAAAAASAAAAAEAAABIAAAAAQAAAP/Y/9sAhAAGBAQEBQQGBQUGCQYFBgkLCAYGCAsMCgoLCgoMEAwMDAwMDBAMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMAQcHBw0MDRgQEBgUDg4OFBQODg4OFBEMDAwMDBERDAwMDAwMEQwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAwMDAz/3QAEACD/7gAOQWRvYmUAZMAAAAAB/8AAEQgAqwEAAwARAAERAQIRAf/EAaIAAAAHAQEBAQEAAAAAAAAAAAQFAwIGAQAHCAkKCwEAAgIDAQEBAQEAAAAAAAAAAQACAwQFBgcICQoLEAACAQMDAgQCBgcDBAIGAnMBAgMRBAAFIRIxQVEGE2EicYEUMpGhBxWxQiPBUtHhMxZi8CRygvElQzRTkqKyY3PCNUQnk6OzNhdUZHTD0uIIJoMJChgZhJRFRqS0VtNVKBry4/PE1OT0ZXWFlaW1xdXl9WZ2hpamtsbW5vY3R1dnd4eXp7fH1+f3OEhYaHiImKi4yNjo+Ck5SVlpeYmZqbnJ2en5KjpKWmp6ipqqusra6voRAAICAQIDBQUEBQYECAMDbQEAAhEDBCESMUEFURNhIgZxgZEyobHwFMHR4SNCFVJicvEzJDRDghaSUyWiY7LCB3PSNeJEgxdUkwgJChgZJjZFGidkdFU38qOzwygp0+PzhJSktMTU5PRldYWVpbXF1eX1RlZmdoaWprbG1ub2R1dnd4eXp7fH1+f3OEhYaHiImKi4yNjo+DlJWWl5iZmpucnZ6fkqOkpaanqKmqq6ytrq+v/aAAwDAAABEQIRAD8APkTJKqquKrwMKuOKomU/uj/q/wAMtamLaavxOf8AKP68qb06iG2SYlEoMLFXUYqqAYqibYUST3GSixkx+Jf9Nm/1zkWfRH8dsLFSYEOp/wAofrwqn88lHOBCmJMVXq5xVUD4pb5jArg4riqoG3xVVR8VVkfFVdJMCoiN8UoqN8VRET7YFRKPiqqsvvgSqCTFXF8VU2fFX//QkarklXgYq2cKpH5t8xjQNIfUTAbgJJHH6Qbif3jca1IPTFWLS/nMihFOlN+8iVx++HRxX+XLOJhSXwfmjFAvI6YxDHr6v/NmQpnxI2L83oP+rY//ACMP/NGFFoyH82oWH/HOYfORv+qeFFoyL804G/48f+Sjf9U8VtEr+ZkZ6WBbv8Lsf+ZeNItFab+ZMd5EZLWx9aMkqXSQkAqaEH4OoPbJBBVNO1S6ubmVhbKhrUhnYdfmmCk8SHfzBrQkm3tkiid15Mj7KjEVJ5jwyNlnw7JV/wArFQqWM8VFO5+qz02Pb48u8Gfc0+NDvW3v5z2ltKyTzRiRdiBaXB/U5yBhIMhKJ6oI/ntYA/DNGf8AozuP+a8juyoJhp/5sajqLBbCOGQnpyt5UH4yZKMJFiTEMmjvPzIlhEsUOm8W3AJkr93LLfy0/Jr8eHmx7XPPfnjRrkW19BaRyMvKNhG7Iw/yW57075TOMomi2wIkLCVW35teaXv4IStpwkcK1InrQ/8APTIcTPhT0/mbr8fWG2b/AGLj/jfCwTjyh581PWdYayuLeFIxC8vKPkDVWUU3J/mwqziOY4qiElxVExPgVFxvilEI+BVdJMVVFkxVUEmBLvUxVaZMUP8A/9GTDJq7FWicVYV+a5/51Cb/AIzwf8nBipeS3xcPamQ1H1WDhvX4eOwHhhYqSOWap+gYqjIK4UJhBthVHwDChNrI8WHhhVUksrzTbltW0lPU50OoaepoJ1H7adlnUf8AIz7D/ssrS2y/Qryx1Zba5spqpPsrd1Kn4lZD0dSOLKw5LhQ8+/MjUdR0q1iewIU3NxKtwjglWVKkCldt/wCXBCwbHNM6MaLFdd806hHem0WC24JFAAxjdmNYUJ5ESKvfsuWDVSGzWdNG7S06vbXk0kmoBgW3Bt4gTX35zLgOe+f4+1PhVy/H2L4otBlkAWW6Vj0HoxD9cpyPGngLJ/LuuaZp0itHJdOi/smKEA/M865OOWipgXo8HnOWIPFJFPBLGnqGOZAhC0DfzHqDUZfg1sJ1w7gteTTkAkoPVvMFhrdgbW+QhTVreelCrjbkhPXwbMvJiExRcaGQxNhgMULQa5bxMQxWVaMOhHY5p5wMZUXZRmJCwySZcDFkP5Zj/nZpP+YWT/iaYQpeqAkYUKqSHAqLhkxSjInwKiFkxSqrJgVUWTFV4kxV3qe+KrTJir//0pLk1bxVa1cVYV+bI/506f8A4zwf8nBiryC7JLQf8YIqf8AMLFuEUocKoyE4oZB5Z0xdV1mz055DEt1II2lVeZUUJJC1FemSAtWV+aPJtnoenWF9a3st0l47IUmh9Fk4qG3HJj36HDIUSLumzLhlCuIVxBKrXti0pzZOVI8MKofyk/pfmHqsUXwQNFaytENlMjCQM/HpyIVanAOaeiSfmVF6lpZqRT/SJzSlMswiyWObkGIaV5J1TXDLfTzNbKLRr1JXhYpKkR4UUgqKtT7WarW6zwKJiZccxj/0/wDE5WPHxfLias/Ieo3GiXWqq0itbzx25smt5PWdpeJBUVr+104YZ6rhzxxUfXEz4/4fT/CgQuJl3K1z5Hv7TR7LVPVMqXnqEwpC/OJYjRmc1Pw/5VFxw6wZM08QBEsXD6v53GssdREv5ybyeTLrTNZsLGSdJ2ulglDBGChZnoAwqT23yrT9oRzYp5IiQ8Pjj/S/dspYjGQHeyrzM1/Lrd5b3fpfW44vQkMAZUNFqDRq78WC/wCxy3sTHEY4cHFwyPF6/qYayR9V9yWfVNUuYoLaaRmgtQwt0J2QOeTBfDk25zqhEui4wk81u8HmK2if7SulfpGajVCshdrpjeMMilQ5UzZD+Wi08yy/8wsn/E0xCvTypwocCcVRMLHAqLjfpgSiFfFVRZMUqiyYFXh8Vb54q0XxV//TkuTV2KuOKsL/ADZ/5Q2f/jPB/wAnBirx26PxQf8AGCL/AIiMLFdFhVFxHfFCaaXf3Vjdw3lpIYbmBg8Uq0qrDuKgjCrINT82eYdbSJNVv5LtICWiVwgCltiRxVeuFSXWjdMLFOLV+mFUJ5aen5iaqen+j2n/ADNyPVPRKvzFkK2dh+yTPcDp03G9Mu053LDOPSGZWuq6BB5NmbSJ4buG4NrZKY9zDZJIkUsklQGjWNPUaTkOKccxJTA5t4Hcnk1/pUfl6Jze26NcXUkrT+qnDm0bJGrS141NV4VP8uPELrqqKun0iW60/S4rq2WCOCFKllRJI2ZmlKVP7xDxTlwwCQJI6rTcOowXXm29nldYrS1vQqK5ChlhtYyh4Ehm/eM/Db7WII6JovLPrkz6hq9/c8uQu7xgz1qY/Xb0+v8AxWVzJ0pHHE9Las49Evcr23mK2DA1GdAJxdHwFJtTu4pfMMd4P7sFWNPBVzR60/vS7nSj92EbbeZNKu5RDG55tsAQcx2xmf5cqR5ll/5hJP8AiaYoZj5o856B5YtobrWbgwRXL+lCVjeUswUt9mMMeg64SoSO2/OLyDcB2ivpXEa85CLa4PFfFvg2X3OC00i4fzc8hHpqRp/xhl/5pxtaKKj/ADb8hD/paAfOKX/mnBaaKIT82vIDsFXVkLHYL6ctSfYcMbWm/wDlbn5fg0OsxD2KyD/jXFaZXp+p2t9ZwXlpKs1rcIssEyGqujiqsD4EYoRYlGKVwkwK7nir/9SSVyauBxV2KsM/NkA+Tpv+M8H/ABMYVLxy5PxxDwhj/wCIjFi3EdsKoqM4oRkLdMKplbnYYUJrat0woTe1fcYVQXl16fmDqp/4otf+ZmRHNPRKfzMPHT9N2pWe42Ip38Bk8XMoy8gt/KLT31XT9S06SLnb3NxHZ+sGPNEnUvMiLts6x8v9blmDlxiUxf8AD6nIiaiWY2vkfT7q5udEijk/QNlcSyoXldiRaKRxY9ePruv+xi4ZT4ZOWUuvDUfx/pm248AHmrQ+ULW80g6xfySxxaOiR6akJHE+sQONCCKEN6fCmVaaJEJz/in/ALxnm4eKITrQPKekSeZoNX1X1hLdTnTbGHZuPoxmjGv7RZZfjVvh5ZXlxnHpajt/EmJBypF+ZOhadpemXN3bXM7tq5ubhLaWgWOOPgnJBTkvNvi4kt9rNj2dEiML504uqIPFTyyF09LkG3zfg7OpIRtOcUbjeqN/xE5rNQfWXYYPoDGLLVHsZUmVF5qQRzO1cpZMn8v/AJr+ZtPvGvbTTILglGh3EgWhIJ3Fd/hx4lpX80+etX85QWttrGjC3itZDLE8DSAlmUrvVfA4k2kRSuztYbQTiz+tW/1mMxXARjR0NfhaqHbfFNNCxt0FBFcH7/8AmjAlY0Vuo+OK4HyNP1pihV0+/g069hvbVrmK5gJKOGjJ3BU7MhG6mmKkIa6uLS4uJJ5Xn9SZ2dmPp7sxJPYYq9f8ifmxGmi2+jW+mO7aRaQxNPJMB6gUcOVFU0rSuSYl6+tyaAkUJAxQrRzVxVWDYpf/1ZGDk1bGKuxVhn5smnk6Yj/f8H/E8VLxq6P7yL/jDH/xEYWLcZ2GFUTGcUIuFsKpjbN0woTW1bpiqawN0woS/RGZvPeq8G4MYbWjEVA/vO2Ac09Et/NEcNO0w1ILXFwSD0FPAdF+jJY+ZWfIMn/LPQ9U0XQpbpZ0himtkvZpN0ZJ54ysSGvNZOCvX7P8ua3VxybSgar6v6jk4qOxTezt/MFp5avw15Eour6SG2uwTwljLB5yQRVUd1lpw/ab4crySnHIJf5KQ9X87j/4lnCIlGv4ophf6V5yvvIENxCptwssd29ou4HpyLIkQYBW5ScV+2rcPs/t5i4808WY4pG4Trw/6PH/AMebJQEo8Q5j/er9T1HzHb+YtIaCNJobO6j9S0DIrrM/KScGlVKCNlblxRv8puWWxOWeKcJislGv97/pkUIyEhySL83oNajCyaiKQvZzwWp4lPslWJ4nswH/AAvxfay/srWeLUT9ca4mrV4uEE9HjLO6mlds39urpkdipbS4G/4rf9TZh5fqczH9LCWvJ7UhoX4Nw4k0B2YUI3rlRSF9rp15ql/YWVrb/Wp2towluCqVABY/ESoHj1wxgZGgiUhEWUTd+VNZsv3cunTwztRk9Xgh47g0Ab5ZZ+Wyd33Nfjx70OukeYF+zFMP9WSn6mx/LZP5qfHh3tnTfMQH93c18fUb/mrB+WyfzSvjw70z8qxy2vmC0m12O7fSUL/WkAklJrGwT4FPxUkKnMTXaXUywyGIEZf4P9N/xLZizY+Lc7PTP0v+V7BQI76tNgLW+T4h/qE1BzmfyPbQ6H/Txk5gz6bvDDtYvNJufMOrxaU07aSmizym3uPXAFxGvLmqXBLoVbjwbN92bDURxVqP7y5f6T+H6WjLKJPo+lG/lhcwzJcxC3CXEVuPWuuTFpQ0tUBU/CvpgU+H7WbANJfTcm1PkP1ZJi3C++KotHqMCX//1pHk1bxV2KsL/Nun+DJ6/wC/4P8AiYxV4xcGskX/ABhj/wCIjCxXRnbCqIQ4qi4ThQmFu2KEztX6YVTSB+mFCA0GSnnzUz/xVbfqkwDmk8kv/Nih0jSV+zymuB0Apsew2xid2UuQZd5U8922r+Wpmey+qC0uIJLzgzTApamJwo+FCobb4RzzB1GWqiBfG3Yo9e5NJfOWm3WhabeXNjJZ2kIuIzYyUNw00qUV9hxqU5kCmVTzCWQYwOKvVxfzeH0sxEiJkerIZ/O2gIC11KYkuZLQ2WmKwEjpD6nMgFgH4vw5lC32U/ycqvjziQG0BKP4/rfwsuWOj/Elum6/osHmqU3r+pfXEl1cxogqgidYhGZH6r+7/Z4/F8eWY9RAiWXfh26LKJoR6sV/M+/vru3Elxc/WEttBQD4w4S5eVhP06P8EYav8uHsuERKRAr1/wCw/hRqjcQP6Lxpp3JrXN3xOupmuk1by9buf99Sf8bZjT5t8OTz+/Oy+NBXIFITvy0ANac9ktEWnsyJUfrzofZmF6gk9If76LrO1pViH9ZlRkVUbioGx7DO58OHUD5PPCcu972Pyx8vyCJotJsJIWjQ1cyK4PAVJ4H4iW+LPlfL7d9o8cv30x6pcP7vDw8PF/Tx/wA19M/krTcuCP2qDfll5X5vHPpdvBIKMgSW4IKUNVqW7EL8Q+L4sR7c9pcxl4v+SOm/6pMx2Rpj/B/sp/rSPzZ5D8p6d5U1HU4LFYLu29MQmO5lmH7yUICwY0751Hsf7U67WdqYdPmlHLhy8fHxYcOL+7xTyf5OEP5rq+1uzcGHTynCPDKP9Ocv4ox/il/SecafKscySxVimjNUkQlWU+II3Ge8HQ4f5sXi8eeV82NajO8vmbzVMzF3XSJg7sSzEssK1JO/7eef9swjHVTjEcIjX+5el0ZvGCUd+U5/f6l/zDx/8nDmuDeX1FIdh8h+rJMVqN8WKoyJtsCX/9eR5NXDFW8VYT+bv/KFz/8AMRB/ycGKvFp2+KL/AIxR/wDERhYr4jhVEI2KouFsKEdA3TFUytnwoTOB+mFUt0aSnnXVDX/ddt+p8A5qeSG/NYn9D6KelZrjbYfq2wDmzPIJ1+SGl2wiu7zUJ/QtDcwlkkNI2jVTKDQ7OWeEf8i8xZyjxizu2RvhZ/5V1KwvtSvdZnMcNpFdXvp+oVBLRySQRlQdyWQE1/ysowwAzSP49TfkkTjiue3ih0Ca8uZIXu7z6haWTPwYqsrR1IXotGmb/KbGER4RA/pIlL94D7l2raTFFpEB4xjWNSvDKZioaYQxigVf5QyxqvFf2cObHeKv6q4p1kv3sZ/N2y07SvLiWEFvHHfyWM91qMyAB3keRKcyOpqz9fs5m4xVDucaW9vBDIemX8TTT0HQ9/LFuf8AiqT/AI2yqXNtHJ5zqdRUHYjtkCoZH5eQfpvUSOiJGo+7+zOq9lh+8yH+jF1HbB9Efe910f8AJ/Sr/RdPv2v7tZLy2iuHEccciK0iBiop8Xw175yPav8AwTdTpdXlwDTRnHBlni45TnDjjjlwcf0cPqdnpvZvFkxRnxyucYy/0wTSw/KeOzkWSLVJZVY7RXNpKwHEHY8JY6Vrmi1f/BS8UGMtMMZ/nY88OL/pZp8jnYOwTjO2Ti/rx/4/BGf8q+uUeJV1ChZmccYL5BR60Ulbk8eNcoH/AAQtPIHiwzGw/i0mT6f4vXpo8XE3fyTMfx/9NI/9Pkq1P8rdcunlibzFJ9WkYEWjpdyRihqB8bvWhFfizb6P/gl9m4qkNKfEiP76I00Mn/Svw/8AYuFn7Az5LHingP8AB6pQ/wBlOTFPMvkW68tWtvdvexXcc8xgAjV0IYLy35e2d/7Me2eDtic4YoZMRwxjOXi8H8fp9Phyl/Nef7R7GnowJGQlxHheaTGt950nP7NmkNf+MskK/wDGmaXtk3qsnv8A96Ha6P8Auoo/8rZfTl1JgKn0oFp/rTUzWhvL6mkbZfkMkxUlPxYqjYWwJf/QkQyatjFW8KsK/NwA+TZQf2riAD5l9vxxV4nchkmVHFHRFVl8CooRihdGcUIhDhVFRNihGwthVMLd+mFCYwS0I3xVLdIk/wCdv1Q/8V2/6nwDmnos/NQO+h6Gsa/vDNOqrtuxqANvh6+GBl0emWvlLTtJ8sXMiR+kVjttMovwiVzQOzD9qR2b7bfs5ga7DGURIj1Yzxx/3Lk6aXqr+cmFj5V0qz0ayiaNqarNNeiM0KpGKVpyqQrs4ZqfaZ2zC1emIAzD+9jHg5/w/wDFf0nIwTiZmP8AD/ChvMXlpm1Cx0aGWRZgsc8Mg2eJ5JeURbb4vSWNAqty+FMli0px5K5+LXif5o9bEzjKBP8AN+n/AHqIuPLST+brcWFxIstrL6cwYfuWit0JkPHceq5k9NmXh/ssli0p4JYeIkfwz/j9X/EsJTAqfVgv5rcI4p2jm9b17KZlRSXWOBXUoeR3FWai/wA/+wyzsvLIjhlf7v0+pdXjEaI/ieMlxXNvbgU9D0JgfK9v/wAYpP8AjbIHmzHJ5zeGrqPcZAqGVeVYS+oas46CTiPkrNnYeykd8h/qf750nbJ2j/nM3OraeamTRbPnT7SerHv40D5vv5PydM2Wv6Xhy/6duF+egRvjh/sv1okeZLBWUppbRAfaWO9ulB+XxGmYw7Jy0QcvH5zw4P8Aewi3DtKA5Q4fdkyKsfm6GM1W3vV36LqVyu1OmQn2NKQ+rF/nabFJsHasf5s/+V00QvnQ1kCT6vEpr6fHUpiR0oTXMY+zkSBxQ0kj/F/gmP8Azv4mf8rx33zD/ktJT1jWhq0NvELnUbj0XLcb+dZlFRSq0VTyzK7K7J/KSkeDTY+Ov8Vw/l5en/VPVPiaNXqxmEQDllw/6tITeczMDaed37mWyQf9JQ/5ozi+05cWpyH+m7zTCsY9yZflQaXWp/8AGCL/AJOHMINpfUTnYfIfqybBYp+LAlFwnFX/0ZEMmreKt4VSDzqivpESekJna5iEURVXVpKngGVvhZOfHn/k4hEuTwrzUix67OinkFVK/AIwG4/EFUbcQdlxKAgoztiqujYVRETYqjInwoR0EnTFCPik6YVS7R5P+ds1M/5MH3DlgHNPRd+aQpomiMGJ5TXBAJFBSvTjt92RPNn0Tf8ALvzBq+paPNp8t3JeXdpLHHZWt07yq8k7j0n5tUp6Xxr8L/Y4/BmFqYmZEAaB+puwnh9XczK3ufObXtpZQumr6xprSpPNJJ6MbW4+JloE4r6bqipVPi4fE3xZjkSzT4eLhhw/T/S4g3V4Y4qso19X84jVE1C1gS8vliWW6vDxMUavzSKqFgAxAVm9J/h/ly2EpGRyH6Y3wsCKHB/EaXQeYPMVjq01vBZr9Vdmt7nUX+L/AEq5l9SZI3B/3UGqeSf7P4cY5JQiZy+qZ5fBHBxGh/CwLz5pscOlXl3biU2cOkQ6ZG8y09Q2krK0iP8AZlVuX2lyegxzjE8YFzlx/wCnRqJiRFdI8LyCozPcVn2hSyf4fgT0m9NYGZZgVoSedRQkN8NPDBTK2BgF7y3UitZEqPbkK5AqmGl+ZLnSLi8EUKTCaVi3MkHYkbUzbdm9rz0gIERLiLianRjKQSapMv8AlYVx+1YRfRIw/wCNTm1HtXPrCP8ApnEPZMe9tPzCUPyNigI6UkDD7mWmTHtYeuP/AGf/AB1h/I45iX+xVj+YdvIOL2Zp/kekD94CnLo+1OIfwT/0zXLsiR/iH+lVYvPulD7VpP8AR6Z/42GWj2qw9Yz/ANj/AMUgdjyHUI+3/MHy+Kc47hP9gD+pjk4+02nPMTHwZ/yZMdQkkE6zeXPNd2tfTub6y9MnY0M00lD/ALHjnE6nIJ5JSHKU5S/2TuccaiB5J1+VbD65qY/4oir/AMjDlYSX1Ax2HyH6smwcvXAlExYq/wD/0pFlit4q6uKsJ/N1mHk2VlNCtxART2fFBeH3UkkkwkkYs7qpZj1JIxVfGcUKynCqvG2KoqJsUI2GTCqNikwoS/SZKeaNSP8Akw/qbIjmnoifzSNdA0E/8W3Hh4n+X4f+ByJZ9GTflDbyaNaT3k9k9w8sMWpwo/7tTGqSKtGIKnmT8APH7WYOpz+HOJI2l6OJuxx4gQObLNK80wR2Osa2YJTdXNbcilGhlnJPF4/t/uua8yvL4cjizxGYwP1S9cf6n0s8kSYgjorXmv6FZ+Wbe2tAyjVLu0RpqqEaGJ4lk4kH4hQPVjxyGHPCWOUB9WP0yUiXEJd6J1y/0d7LRtDhlYTNM17NVCppKr8Gpu1Cf5eXJlyc8uOeESB9IpOPiEz7ikH52X0D6E+mWb87LTLD0wwp/eu4DAjqrKqJ1+L48z4SBFjk4pD54brkmLPtJYr5VgI6+i//ABtiyYP6FwZ4yg/eKQVr0qDUZFCa6f5euNRumhisS0xBkIS4CClRX7Ub92w0tou40CTQJYLu+S6sPUYpDLHLDLVgKkfYXt7YCFIB2KbRavrLwF7bVpxAsZlZpYLWQCMdWNUG304OENR08O5uxbXNUvLe0jvbS6e7JEZuNNsylACWYsoJooViceFfAj0v5ySPUora5j9JntYZKhjJb6e8R+XKPb8MNM4wrqUu/QiE0W/gLHorJcKf+TVPxxpmnEUUFn5Ul00zJPeXd9HcMIuRVIYYmUcmZV+JnbZf5cQkimSfl3dySNPYiOL/AEWGkZiSkzmWXkRIQSXpT4NvhyQYF9LLGxVSRTYZJgvVKYpVkFMCv//TkIyat4UNHFWFfm6f+dMm/wCM8H/E8QgvDZvtL/qL+rFK+M7YqrIcUK6NhVERvihFRvhVFRSAU3xVAaY9fMOo79RD+HLAOapl+Z/F9A8vqzcVaWcMwoaAnc0XY/7HIyZ9HrVlrOhXPlcpod3Fctf3FpbD0QweO0R0Ry/IBl4xh/2eKtlGpnEQNlniviCbJBDLo9la2t3E08rTT3EyujcpJmCUMn2eVJK7fyrlU4AiA7j+hsjOrSrVfL2m3/neHQrOJH0+0tYLe4VQGQoavIN9wOIHJ/8ALwmFZgR/W/0qiX7sp3pOhafr/mxS1tGbCyupZI5ANwtnSNVDfsoJd+KnK8OniDOAH7v+Z/D6x6kzn6Ynq8d88y3t/NrMUZ9QQ2L3Ez7l5RLKxQjf9lIyWr/k8cs0cSIkdLPD/mrqCLFdzyU75luK9C8vUbQ9PQ7hgAR82OEMuiMu9Mt1NRGtR3oMLBM/y9sBJ5kcU2FtIf8AhkwhBeg6r5T0nU7Ex31kl4IQ0kET1+3xNKEeOEhALx5dH1yK3lh+pyRxzoEkR7eVaKCG4jbbpldNto3y9bTWt9MJk4XFxbmysVVSqq0pCN1AofT5Kv8AxkwhXoTfkt5fkAPr3SyEDmyutOVN6BlOS4WHEp2/5KWFpew3tnql3FPA3KMssDjcFSCClCCpIxpbQV3+RKzzPP8Ap24MrkszSRqdya/slcHCkzJ5vQvLfl610iwsbKMLJLawxwNdFFEj8AByYjf4qYQxZaq7dMVdxGKuAwK//9SQZYhvFWjirCfzeP8Azpk3/MRB/wASxQ8NlPxL/qr+rAlehwoVVbFVVGxVXRsKq6SYoVo5CDhVCaXJ/uevj4iP9RwDmnonH5nEHQPL/f4599j3/wAn4fuyJZdGRflDpT61p6acFeOKZ5Ip50YqxTmJHZCpBBC/By/Yb7OYeTFxZRe4+pyIyAx+bKdN8n6Jq6toUTTL5fgup1uJWcESQWLiMRsRQ8VlA5P9rhF9vK5wl4k5geqMfR+P9Mo4eEDvPqZBrfkl5rm6u4dWeGx0iBKsgNZJJaqq7cXRlQoF4P8AyZi6AeiWYj1z9X+lDbmHqEAdkFFaa3HOurJqptNL9YWMEBLIZTyDSTSBT6cnNlb7cfLjy+P4syeE48JIJ4p/77/iWsDinXSLEfzE8tz2PlG91+VUiOrxNFZiNiGFrbv8IdPsrX1OXw/zccysGMwiLN/8U1ZJcReFk5e1PQfLbf7itNHuv/EsIT0ZDdqCTkmtOPy0hB8zSbf8esn/ABNMQpeppGBk2K+tOmBVyqjGpAJ8TilFxKDgVVKCmKVJkxVfbx/HXwxVMlG2BW6YFW4q/wD/1T+uWIbrirROKsJ/N4/86ZL/AMxEH/EsUPDZftj/AFR+rAltDthVUBxQqq2KqyNhVVV8VVFk3xQoaQ8Y127MgJQ+nyCkA036Eg4BzSnX5lq7aFoBUmRnebgood60AXiN+WCTLo9J8neW7/ynZSS28p+G3SK4NeHK7kUlwKV5Rp25cfi/azX6sTjKM4yrf1R/nR/muTgAkDEhW0O0816L5LEXrwvJc3U0Mc8tB60EjCSQ/stG2z/Z5ry+Lg32MEssxMSr91kj/nRyf8SoxjeP8UE/1nXfMlx5dNxa2QgsZ57fULqFkIn9CN43oxBZXkKoSirxbMTT5pY70865cOI/z+L+L/TNk4cX7wcv4lDVdXmOo6VpM1l6NrbPyLxcqCe5SSNUk5Asknx8v2lzIGpM8JJiYyh9WP8Ai9DWIVLyLG/zm1ZL3QJba3i9O106yeA8TzX1GeMmrj4S3wf8NmbgzjJEEbbfS0zgYl89E75c1s/8vN/uM0z5r/xLCEnkyS4bc5NrZD+WQH+JZP8AmFk/4mmEKXpzUFckxUmO+BVaLFUZCMCURTbAlYVxVVgSmKotemKuJwKsJxV//9Y8DZNC/CrROKsI/N8/86XL/wAxEH/EsUPDJD8Q+Q/VgSuU4qvBwqqKcUKqtiqqGwquV98VQ+mvTVro/wCp+o4BzVk/n++ltdN8r3kPFpbeaSePnR1LRuGXlSgYVG9MEmTP9N89X3mHytZtJaxafFbO97qIi5MJk/eRihYlhydlkC/HmDq8hI4IjiN/6VydPGjxHYI+985aBqegaXdT272enW6uPTmKPIZZkHEihCFxSSP0yY25Yc2QGQx0b9Mv6LDHYBkyj/FOnyS3E0l6bLQ/9DRIXqHBjMpl5pTkK8I+Vfg+D7XHMTIIZNXAgbwEr/zfpboEjCfggtIeyu/OFzqV/drF/pM89nbyMtXVI1iiMY/a+Fmb/Z5l4pQlklIG9g1yJEAC81863Us/lnUVkiEBe2M7KVKuGMuyknfoeh/mwaWAuRBtOaRoB4wTma4rPfL5/wBxumfNf+JYQnozTUb2xk0e0tY4FS8hklaeZVoWVvsgt1b/AI1yXVgmX5ZH/nZJP+YWT/iaYQxL05jvkkKZO+Kq8OKUbFgVEdsCWqYqrxjFVXFWicVU2OKv/9c72rk0LsKuJxVg35wH/nTJP+YmD/iWKHhrncfIYEtqcVXht8VVFbChUVsVXh8VXK2KofT2/wBydyf9X+OI5qyP8yG5aF5fNa19c1qDWp8RtgLJl/5KzadNb2o1W5jihtpmMMctKSen8aqAdiVdsxhEeKT5N5kfDA82c6BPp+pPe6zemCWyhF7cJZsFoD6kkaj0+pbgh5ch9pnxxR/eSPu/3KJn0gKEOkWjeX5dZ1G0hmuII7eDS6fCqy3DKWMZFD8TTBWZf2VyvFAjHLv9TPIQZju9KJl0e2isE1ee3d728vhHGitRFt7UbgA7UpESW+3/AJWQnjrDt/FX+yWJBnuk35seW49N8ies7v8ApTV0luZLU0McSclCrGN2AHNFpyzLx4owFAU0SkTzfPb6bcqKlDTLKYsw0IFLHTlOxBWv/BYQpZJcdTk2tkP5aH/nZJP+YWT/AImmIUvTid8mxW98CoiLtgSjYsVRHbAlsYqqocVX8sVWlsCqbE4q/wD/0DsDeuTQ3hVonFDBvzfP/OnOKV/0mDYf6xxV4fMjoVLKVDAFa9xgStBxVeGxVcGxVeHwoXh8VbMqopZjRR1OKrNNVvWkuT8KykcQetADvgCSyT8xyDoHl41rUTb1B7+IxKUu8rQta+a7fTbofWIZC8E0GxRlkSrfC/w/sj/gcpz2IEjm2Y6MgCifLusmW61B53kkt1tria3bq8SRO0yHx/bbn/Nz+LIzuIBHMyCx3O6P07zNqI8tXN1NK31m3ktyLZSRHKCYolRkrwqOAZWpyVuWAjhIgOUuJI3Bl1DJv8eatHb6fPNcyTyNO0C2zEuY5ZklowqpJjCn7Dc0XCRZ4O7hUbepF+dvOkuqPAmpTC4le2McRFBRY5QW+EfD2o1OOTx5BIkfzWMocPxYlJfac0IjPHitSBQA79anqcvJ2prrdThaMyWpi+xzXj/wWBJTu56nJNafflq3/OySf8wsn/E0xCl6dWpyTFsYqiIu2BKNiOKq/bAlcuKqi4q3XFWicVU2O+Kv/9E6ByaG64ULWxVgf5xN/wA6ew/5eYf1nFXji3PwrBdqWtyq8aABk2+F0+j/AIPAlQuLd4HAJDo4rFKv2WXxH8V/ZxVYDiq4EeOKrgw8cVXjlStD9xwoclle3VJTbyfVgaJ8DUYjx2wJRgha3kQ3iPFHUFqAc6UrtX54UMz82eWL++8v2Y2lutMDlrYEUkBNHVXAB5bcl2xLJgFr5iFvrserejyljcsYS/coU+1QHv8Ay5VMcQplE0bVLa+0nTYp0t55btrmymtGrCIvTaXj8W7tyAocZxsD38SxNWiLHWNOTSL20aRkmnks2jqppSCRmepFex2xlG5RP83iWJoHzpkVtqGmXFtpYS7iElveTSygsFYRvAIwd6ftHERPiE/0V4hw0n3mtbC5v7rUbBFSxl07igqlEdbltjxJ+J04s2Y3Z+LJGPDPefF9X85t1EgTY5UwdoXlYJEA7NsArDNgcZDjCYKa2sRge0hJBZHQEjpUtXIsiyC5HXJNadflxt5lf3tpP+JpiFL1JVOSYr+OKq8a4EouLFVcYErlxVeDirZOKrScVWMcCv8A/9I3ByaF1cVbwoY3558r3HmPRv0bbzpbuZo5PUdSwohO1ARjS2w4/kfcx2/K51WE+kCSUt25H2JaU9KbbZLgRxLrf8pbK5gRX1N1j2PpxwxgVApy3r8R7nI0lFxfkhoWxfUrw+yiBf8AmWcPCto2P8l/Kqj45rt/+eir/wARUYaRaJj/ACh8np1S6f53Mo/4iRjS2i4fyx8nxCgs5GH+XcTt+t8aW0W/5eeTltiRpMLv+zzLtv8ASxyXCKY3up2fkbynHQyaHZFvEwqT+IwcKbVp/JVjLK8seoXlu8jFiEdCoJNdlZCAMeFPEll9+Wlo8Mj/AFpJyATS5tIHr8yoTAYpE0il/KuGTcW+nP8AKCSE/wDCOcjSbQE/5QOSSlhAfeO8mQ/8C6kYrsgJ/wApr6MHhY3f/PGe3k/4nxOG0bJbcflxqkIJEF9H48rYSf8AJpjXDa0u0/S4tKhb1Y5/rLfbmlt5YtvABl2GApCnHeWkmoQKk6MwlSqhhX7Q7YKW2faR5Q1rWGDxRehak73MwKqR/kj7T/R8P+VkmDP/AC75M0vRGM0Zae8ZeDzvtsSCQqjZRthAQnnBfDFWigxVUQYqrx4qrA4ErgcVXA4q4nFVpOBVpOKv/9MyDDxyaFwceOKrhIMVXxsPUX55IIKIvWWSJ4RvyFCcsLWEug0+KFQFBoMFMrRSIB2ONItUCjxpjS236f8AlYaW1whr+1jS2qLCKUJrhpCosEfhhpCosCY0tunhQwOtOopgPJQhksxTplbYqiz9sVXC09sUL1tiO2Kqq2pYUIqPfCq1tG052Dy2sUjqaqWRSQR33GKEYF7Yqu9IlSeww0hTK4ErSuKrlGKqq4qqg4FbBxSuDYq4tiq0nFVvLFX/1BZAyxi2AMVXBVw0qrGq8hthAQigTkmC4YVbwq7FW8ULhiq9cKqgJphVepOKFx3/AAwHkkIlVXwypmqBV8MVXcV8MKr1RfDFC+gA6YqtOKuGFVSL7DZIMSoEZBksOKuGKqi4qvxVvAreKuPTFVpxVacUv//V/9n/4gxYSUNDX1BST0ZJTEUAAQEAAAxITGlubwIQAABtbnRyUkdCIFhZWiAHzgACAAkABgAxAABhY3NwTVNGVAAAAABJRUMgc1JHQgAAAAAAAAAAAAAAAAAA9tYAAQAAAADTLUhQICAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABFjcHJ0AAABUAAAADNkZXNjAAABhAAAAGx3dHB0AAAB8AAAABRia3B0AAACBAAAABRyWFlaAAACGAAAABRnWFlaAAACLAAAABRiWFlaAAACQAAAABRkbW5kAAACVAAAAHBkbWRkAAACxAAAAIh2dWVkAAADTAAAAIZ2aWV3AAAD1AAAACRsdW1pAAAD+AAAABRtZWFzAAAEDAAAACR0ZWNoAAAEMAAAAAxyVFJDAAAEPAAACAxnVFJDAAAEPAAACAxiVFJDAAAEPAAACAx0ZXh0AAAAAENvcHlyaWdodCAoYykgMTk5OCBIZXdsZXR0LVBhY2thcmQgQ29tcGFueQAAZGVzYwAAAAAAAAASc1JHQiBJRUM2MTk2Ni0yLjEAAAAAAAAAAAAAABJzUkdCIElFQzYxOTY2LTIuMQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAWFlaIAAAAAAAAPNRAAEAAAABFsxYWVogAAAAAAAAAAAAAAAAAAAAAFhZWiAAAAAAAABvogAAOPUAAAOQWFlaIAAAAAAAAGKZAAC3hQAAGNpYWVogAAAAAAAAJKAAAA+EAAC2z2Rlc2MAAAAAAAAAFklFQyBodHRwOi8vd3d3LmllYy5jaAAAAAAAAAAAAAAAFklFQyBodHRwOi8vd3d3LmllYy5jaAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkZXNjAAAAAAAAAC5JRUMgNjE5NjYtMi4xIERlZmF1bHQgUkdCIGNvbG91ciBzcGFjZSAtIHNSR0IAAAAAAAAAAAAAAC5JRUMgNjE5NjYtMi4xIERlZmF1bHQgUkdCIGNvbG91ciBzcGFjZSAtIHNSR0IAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZGVzYwAAAAAAAAAsUmVmZXJlbmNlIFZpZXdpbmcgQ29uZGl0aW9uIGluIElFQzYxOTY2LTIuMQAAAAAAAAAAAAAALFJlZmVyZW5jZSBWaWV3aW5nIENvbmRpdGlvbiBpbiBJRUM2MTk2Ni0yLjEAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAHZpZXcAAAAAABOk/gAUXy4AEM8UAAPtzAAEEwsAA1yeAAAAAVhZWiAAAAAAAEwJVgBQAAAAVx/nbWVhcwAAAAAAAAABAAAAAAAAAAAAAAAAAAAAAAAAAo8AAAACc2lnIAAAAABDUlQgY3VydgAAAAAAAAQAAAAABQAKAA8AFAAZAB4AIwAoAC0AMgA3ADsAQABFAEoATwBUAFkAXgBjAGgAbQByAHcAfACBAIYAiwCQAJUAmgCfAKQAqQCuALIAtwC8AMEAxgDLANAA1QDbAOAA5QDrAPAA9gD7AQEBBwENARMBGQEfASUBKwEyATgBPgFFAUwBUgFZAWABZwFuAXUBfAGDAYsBkgGaAaEBqQGxAbkBwQHJAdEB2QHhAekB8gH6AgMCDAIUAh0CJgIvAjgCQQJLAlQCXQJnAnECegKEAo4CmAKiAqwCtgLBAssC1QLgAusC9QMAAwsDFgMhAy0DOANDA08DWgNmA3IDfgOKA5YDogOuA7oDxwPTA+AD7AP5BAYEEwQgBC0EOwRIBFUEYwRxBH4EjASaBKgEtgTEBNME4QTwBP4FDQUcBSsFOgVJBVgFZwV3BYYFlgWmBbUFxQXVBeUF9gYGBhYGJwY3BkgGWQZqBnsGjAadBq8GwAbRBuMG9QcHBxkHKwc9B08HYQd0B4YHmQesB78H0gflB/gICwgfCDIIRghaCG4IggiWCKoIvgjSCOcI+wkQCSUJOglPCWQJeQmPCaQJugnPCeUJ+woRCicKPQpUCmoKgQqYCq4KxQrcCvMLCwsiCzkLUQtpC4ALmAuwC8gL4Qv5DBIMKgxDDFwMdQyODKcMwAzZDPMNDQ0mDUANWg10DY4NqQ3DDd4N+A4TDi4OSQ5kDn8Omw62DtIO7g8JDyUPQQ9eD3oPlg+zD88P7BAJECYQQxBhEH4QmxC5ENcQ9RETETERTxFtEYwRqhHJEegSBxImEkUSZBKEEqMSwxLjEwMTIxNDE2MTgxOkE8UT5RQGFCcUSRRqFIsUrRTOFPAVEhU0FVYVeBWbFb0V4BYDFiYWSRZsFo8WshbWFvoXHRdBF2UXiReuF9IX9xgbGEAYZRiKGK8Y1Rj6GSAZRRlrGZEZtxndGgQaKhpRGncanhrFGuwbFBs7G2MbihuyG9ocAhwqHFIcexyjHMwc9R0eHUcdcB2ZHcMd7B4WHkAeah6UHr4e6R8THz4faR+UH78f6iAVIEEgbCCYIMQg8CEcIUghdSGhIc4h+yInIlUigiKvIt0jCiM4I2YjlCPCI/AkHyRNJHwkqyTaJQklOCVoJZclxyX3JicmVyaHJrcm6CcYJ0kneierJ9woDSg/KHEooijUKQYpOClrKZ0p0CoCKjUqaCqbKs8rAis2K2krnSvRLAUsOSxuLKIs1y0MLUEtdi2rLeEuFi5MLoIuty7uLyQvWi+RL8cv/jA1MGwwpDDbMRIxSjGCMbox8jIqMmMymzLUMw0zRjN/M7gz8TQrNGU0njTYNRM1TTWHNcI1/TY3NnI2rjbpNyQ3YDecN9c4FDhQOIw4yDkFOUI5fzm8Ofk6Njp0OrI67zstO2s7qjvoPCc8ZTykPOM9Ij1hPaE94D4gPmA+oD7gPyE/YT+iP+JAI0BkQKZA50EpQWpBrEHuQjBCckK1QvdDOkN9Q8BEA0RHRIpEzkUSRVVFmkXeRiJGZ0arRvBHNUd7R8BIBUhLSJFI10kdSWNJqUnwSjdKfUrESwxLU0uaS+JMKkxyTLpNAk1KTZNN3E4lTm5Ot08AT0lPk0/dUCdQcVC7UQZRUFGbUeZSMVJ8UsdTE1NfU6pT9lRCVI9U21UoVXVVwlYPVlxWqVb3V0RXklfgWC9YfVjLWRpZaVm4WgdaVlqmWvVbRVuVW+VcNVyGXNZdJ114XcleGl5sXr1fD19hX7NgBWBXYKpg/GFPYaJh9WJJYpxi8GNDY5dj62RAZJRk6WU9ZZJl52Y9ZpJm6Gc9Z5Nn6Wg/aJZo7GlDaZpp8WpIap9q92tPa6dr/2xXbK9tCG1gbbluEm5rbsRvHm94b9FwK3CGcOBxOnGVcfByS3KmcwFzXXO4dBR0cHTMdSh1hXXhdj52m3b4d1Z3s3gReG54zHkqeYl553pGeqV7BHtje8J8IXyBfOF9QX2hfgF+Yn7CfyN/hH/lgEeAqIEKgWuBzYIwgpKC9INXg7qEHYSAhOOFR4Wrhg6GcobXhzuHn4gEiGmIzokziZmJ/opkisqLMIuWi/yMY4zKjTGNmI3/jmaOzo82j56QBpBukNaRP5GokhGSepLjk02TtpQglIqU9JVflcmWNJaflwqXdZfgmEyYuJkkmZCZ/JpomtWbQpuvnByciZz3nWSd0p5Anq6fHZ+Ln/qgaaDYoUehtqImopajBqN2o+akVqTHpTilqaYapoum/adup+CoUqjEqTepqaocqo+rAqt1q+msXKzQrUStuK4trqGvFq+LsACwdbDqsWCx1rJLssKzOLOutCW0nLUTtYq2AbZ5tvC3aLfguFm40blKucK6O7q1uy67p7whvJu9Fb2Pvgq+hL7/v3q/9cBwwOzBZ8Hjwl/C28NYw9TEUcTOxUvFyMZGxsPHQce/yD3IvMk6ybnKOMq3yzbLtsw1zLXNNc21zjbOts83z7jQOdC60TzRvtI/0sHTRNPG1EnUy9VO1dHWVdbY11zX4Nhk2OjZbNnx2nba+9uA3AXcit0Q3ZbeHN6i3ynfr+A24L3hROHM4lPi2+Nj4+vkc+T85YTmDeaW5x/nqegy6LzpRunQ6lvq5etw6/vshu0R7ZzuKO6070DvzPBY8OXxcvH/8ozzGfOn9DT0wvVQ9d72bfb794r4Gfio+Tj5x/pX+uf7d/wH/Jj9Kf26/kv+3P9t////7QBmUGhvdG9zaG9wIDMuMAA4QklNBAQAAAAAAEkcAVoAAxslRxwCAAACAAQcAjcACDIwMjYwMTIyHAI8AAsxMTU0MDQtMDUwMBwCPgAIMjAyNjAxMjIcAj8ACzExNTQwNS0wNTAwAP/hl5NodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvADw/eHBhY2tldCBiZWdpbj0i77u/IiBpZD0iVzVNME1wQ2VoaUh6cmVTek5UY3prYzlkIj8+Cjx4OnhtcG1ldGEgeG1sbnM6eD0iYWRvYmU6bnM6bWV0YS8iIHg6eG1wdGs9IkFkb2JlIFhNUCBDb3JlIDcuMC1jMDAwIDEuMDAwMDAwLCAwMDAwLzAwLzAwLTAwOjAwOjAwICAgICAgICAiPgogPHJkZjpSREYgeG1sbnM6cmRmPSJodHRwOi8vd3d3LnczLm9yZy8xOTk5LzAyLzIyLXJkZi1zeW50YXgtbnMjIj4KICA8cmRmOkRlc2NyaXB0aW9uIHJkZjphYm91dD0iIgogICAgeG1sbnM6eG1wPSJodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvIgogICAgeG1sbnM6YXV4PSJodHRwOi8vbnMuYWRvYmUuY29tL2V4aWYvMS4wL2F1eC8iCiAgICB4bWxuczpleGlmRVg9Imh0dHA6Ly9jaXBhLmpwL2V4aWYvMS4wLyIKICAgIHhtbG5zOnBob3Rvc2hvcD0iaHR0cDovL25zLmFkb2JlLmNvbS9waG90b3Nob3AvMS4wLyIKICAgIHhtbG5zOnhtcE1NPSJodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvbW0vIgogICAgeG1sbnM6c3RFdnQ9Imh0dHA6Ly9ucy5hZG9iZS5jb20veGFwLzEuMC9zVHlwZS9SZXNvdXJjZUV2ZW50IyIKICAgIHhtbG5zOnN0UmVmPSJodHRwOi8vbnMuYWRvYmUuY29tL3hhcC8xLjAvc1R5cGUvUmVzb3VyY2VSZWYjIgogICAgeG1sbnM6ZGM9Imh0dHA6Ly9wdXJsLm9yZy9kYy9lbGVtZW50cy8xLjEvIgogICAgeG1sbnM6eG1wRE09Imh0dHA6Ly9ucy5hZG9iZS5jb20veG1wLzEuMC9EeW5hbWljTWVkaWEvIgogICAgeG1sbnM6Y3JzPSJodHRwOi8vbnMuYWRvYmUuY29tL2NhbWVyYS1yYXctc2V0dGluZ3MvMS4wLyIKICAgeG1wOk1vZGlmeURhdGU9IjIwMjYtMDItMTJUMDQ6MTE6MTArMDY6MDAiCiAgIHhtcDpDcmVhdGVEYXRlPSIyMDI2LTAxLTIyVDExOjU0OjA1LjEzMS0wNTowMCIKICAgeG1wOk1ldGFkYXRhRGF0ZT0iMjAyNi0wMi0xMlQwNDoxMToxMCswNjowMCIKICAgeG1wOkNyZWF0b3JUb29sPSJBZG9iZSBQaG90b3Nob3AgTGlnaHRyb29tIENsYXNzaWMgMTUuMS4xIChNYWNpbnRvc2gpIgogICB4bXA6UmF0aW5nPSIzIgogICBhdXg6U2VyaWFsTnVtYmVyPSIxNTIyMDI0MDAzMDEiCiAgIGF1eDpMZW5zSW5mbz0iOTAvMSA5MC8xIDAvMCAwLzAiCiAgIGF1eDpMZW5zPSJUUy1FOTBtbSBmLzIuOCIKICAgYXV4OkxlbnNJRD0iMTI3IgogICBhdXg6TGVuc1NlcmlhbE51bWJlcj0iMDAwMDAwMDAwMCIKICAgYXV4OkltYWdlTnVtYmVyPSIwIgogICBhdXg6Rmxhc2hDb21wZW5zYXRpb249IjAvMSIKICAgYXV4OkZpcm13YXJlPSIxLjIuMCIKICAgYXV4OklzTWVyZ2VkSERSPSJUcnVlIgogICBhdXg6TGF0ZXJhbENocm9tYXRpY0FiZXJyYXRpb25Db3JyZWN0aW9uQWxyZWFkeUFwcGxpZWQ9IlRydWUiCiAgIGV4aWZFWDpMZW5zTW9kZWw9IlRTLUU5MG1tIGYvMi44IgogICBwaG90b3Nob3A6RGF0ZUNyZWF0ZWQ9IjIwMjYtMDEtMjJUMTE6NTQ6MDQuMzktMDU6MDAiCiAgIHhtcE1NOkRvY3VtZW50SUQ9InhtcC5kaWQ6NjQxNzg4YjItNDg2Yi00ZDkxLWFjMWEtNDI4NTE0ZDM3YjE5IgogICB4bXBNTTpQcmVzZXJ2ZWRGaWxlTmFtZT0iSFNodF8wMTcwLkNSMyIKICAgeG1wTU06T3JpZ2luYWxEb2N1bWVudElEPSIzOEU2MEY4M0EyRDYyQkRDQzRCQTdEMTZEMkM1Q0QxOSIKICAgeG1wTU06SW5zdGFuY2VJRD0ieG1wLmlpZDo2NDE3ODhiMi00ODZiLTRkOTEtYWMxYS00Mjg1MTRkMzdiMTkiCiAgIGRjOmZvcm1hdD0iaW1hZ2UvanBlZyIKICAgeG1wRE06cGljaz0iMCIKICAgY3JzOlJhd0ZpbGVOYW1lPSJIU2h0XzAxNzAtSERSLmpwZyIKICAgY3JzOlZlcnNpb249IjE4LjEiCiAgIGNyczpDb21wYXRpYmxlVmVyc2lvbj0iMjY4NDM1NDU2IgogICBjcnM6UHJvY2Vzc1ZlcnNpb249IjE1LjQiCiAgIGNyczpXaGl0ZUJhbGFuY2U9IkFzIFNob3QiCiAgIGNyczpJbmNyZW1lbnRhbFRlbXBlcmF0dXJlPSIwIgogICBjcnM6SW5jcmVtZW50YWxUaW50PSIwIgogICBjcnM6RXhwb3N1cmUyMDEyPSIwLjAwIgogICBjcnM6Q29udHJhc3QyMDEyPSIwIgogICBjcnM6SGlnaGxpZ2h0czIwMTI9IjAiCiAgIGNyczpTaGFkb3dzMjAxMj0iMCIKICAgY3JzOldoaXRlczIwMTI9IjAiCiAgIGNyczpCbGFja3MyMDEyPSIwIgogICBjcnM6VGV4dHVyZT0iMCIKICAgY3JzOkNsYXJpdHkyMDEyPSIwIgogICBjcnM6RGVoYXplPSIwIgogICBjcnM6VmlicmFuY2U9IjAiCiAgIGNyczpTYXR1cmF0aW9uPSIwIgogICBjcnM6UGFyYW1ldHJpY1NoYWRvd3M9IjAiCiAgIGNyczpQYXJhbWV0cmljRGFya3M9IjAiCiAgIGNyczpQYXJhbWV0cmljTGlnaHRzPSIwIgogICBjcnM6UGFyYW1ldHJpY0hpZ2hsaWdodHM9IjAiCiAgIGNyczpQYXJhbWV0cmljU2hhZG93U3BsaXQ9IjI1IgogICBjcnM6UGFyYW1ldHJpY01pZHRvbmVTcGxpdD0iNTAiCiAgIGNyczpQYXJhbWV0cmljSGlnaGxpZ2h0U3BsaXQ9Ijc1IgogICBjcnM6U2hhcnBuZXNzPSIwIgogICBjcnM6THVtaW5hbmNlU21vb3RoaW5nPSIwIgogICBjcnM6Q29sb3JOb2lzZVJlZHVjdGlvbj0iMCIKICAgY3JzOkh1ZUFkanVzdG1lbnRSZWQ9IjAiCiAgIGNyczpIdWVBZGp1c3RtZW50T3JhbmdlPSIwIgogICBjcnM6SHVlQWRqdXN0bWVudFllbGxvdz0iMCIKICAgY3JzOkh1ZUFkanVzdG1lbnRHcmVlbj0iMCIKICAgY3JzOkh1ZUFkanVzdG1lbnRBcXVhPSIwIgogICBjcnM6SHVlQWRqdXN0bWVudEJsdWU9IjAiCiAgIGNyczpIdWVBZGp1c3RtZW50UHVycGxlPSIwIgogICBjcnM6SHVlQWRqdXN0bWVudE1hZ2VudGE9IjAiCiAgIGNyczpTYXR1cmF0aW9uQWRqdXN0bWVudFJlZD0iMCIKICAgY3JzOlNhdHVyYXRpb25BZGp1c3RtZW50T3JhbmdlPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRZZWxsb3c9IjAiCiAgIGNyczpTYXR1cmF0aW9uQWRqdXN0bWVudEdyZWVuPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRBcXVhPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRCbHVlPSIwIgogICBjcnM6U2F0dXJhdGlvbkFkanVzdG1lbnRQdXJwbGU9IjAiCiAgIGNyczpTYXR1cmF0aW9uQWRqdXN0bWVudE1hZ2VudGE9IjAiCiAgIGNyczpMdW1pbmFuY2VBZGp1c3RtZW50UmVkPSIwIgogICBjcnM6THVtaW5hbmNlQWRqdXN0bWVudE9yYW5nZT0iMCIKICAgY3JzOkx1bWluYW5jZUFkanVzdG1lbnRZZWxsb3c9IjAiCiAgIGNyczpMdW1pbmFuY2VBZGp1c3RtZW50R3JlZW49IjAiCiAgIGNyczpMdW1pbmFuY2VBZGp1c3RtZW50QXF1YT0iMCIKICAgY3JzOkx1bWluYW5jZUFkanVzdG1lbnRCbHVlPSIwIgogICBjcnM6THVtaW5hbmNlQWRqdXN0bWVudFB1cnBsZT0iMCIKICAgY3JzOkx1bWluYW5jZUFkanVzdG1lbnRNYWdlbnRhPSIwIgogICBjcnM6U3BsaXRUb25pbmdTaGFkb3dIdWU9IjAiCiAgIGNyczpTcGxpdFRvbmluZ1NoYWRvd1NhdHVyYXRpb249IjAiCiAgIGNyczpTcGxpdFRvbmluZ0hpZ2hsaWdodEh1ZT0iMCIKICAgY3JzOlNwbGl0VG9uaW5nSGlnaGxpZ2h0U2F0dXJhdGlvbj0iMCIKICAgY3JzOlNwbGl0VG9uaW5nQmFsYW5jZT0iMCIKICAgY3JzOkNvbG9yR3JhZGVNaWR0b25lSHVlPSIwIgogICBjcnM6Q29sb3JHcmFkZU1pZHRvbmVTYXQ9IjAiCiAgIGNyczpDb2xvckdyYWRlU2hhZG93THVtPSIwIgogICBjcnM6Q29sb3JHcmFkZU1pZHRvbmVMdW09IjAiCiAgIGNyczpDb2xvckdyYWRlSGlnaGxpZ2h0THVtPSIwIgogICBjcnM6Q29sb3JHcmFkZUJsZW5kaW5nPSI1MCIKICAgY3JzOkNvbG9yR3JhZGVHbG9iYWxIdWU9IjAiCiAgIGNyczpDb2xvckdyYWRlR2xvYmFsU2F0PSIwIgogICBjcnM6Q29sb3JHcmFkZUdsb2JhbEx1bT0iMCIKICAgY3JzOkF1dG9MYXRlcmFsQ0E9IjAiCiAgIGNyczpMZW5zUHJvZmlsZUVuYWJsZT0iMCIKICAgY3JzOkxlbnNNYW51YWxEaXN0b3J0aW9uQW1vdW50PSIwIgogICBjcnM6VmlnbmV0dGVBbW91bnQ9IjAiCiAgIGNyczpEZWZyaW5nZVB1cnBsZUFtb3VudD0iMCIKICAgY3JzOkRlZnJpbmdlUHVycGxlSHVlTG89IjMwIgogICBjcnM6RGVmcmluZ2VQdXJwbGVIdWVIaT0iNzAiCiAgIGNyczpEZWZyaW5nZUdyZWVuQW1vdW50PSIwIgogICBjcnM6RGVmcmluZ2VHcmVlbkh1ZUxvPSI0MCIKICAgY3JzOkRlZnJpbmdlR3JlZW5IdWVIaT0iNjAiCiAgIGNyczpQZXJzcGVjdGl2ZVVwcmlnaHQ9IjAiCiAgIGNyczpQZXJzcGVjdGl2ZVZlcnRpY2FsPSIwIgogICBjcnM6UGVyc3BlY3RpdmVIb3Jpem9udGFsPSIwIgogICBjcnM6UGVyc3BlY3RpdmVSb3RhdGU9IjAuMCIKICAgY3JzOlBlcnNwZWN0aXZlQXNwZWN0PSIwIgogICBjcnM6UGVyc3BlY3RpdmVTY2FsZT0iMTAwIgogICBjcnM6UGVyc3BlY3RpdmVYPSIwLjAwIgogICBjcnM6UGVyc3BlY3RpdmVZPSIwLjAwIgogICBjcnM6R3JhaW5BbW91bnQ9IjAiCiAgIGNyczpQb3N0Q3JvcFZpZ25ldHRlQW1vdW50PSIwIgogICBjcnM6U2hhZG93VGludD0iMCIKICAgY3JzOlJlZEh1ZT0iMCIKICAgY3JzOlJlZFNhdHVyYXRpb249IjAiCiAgIGNyczpHcmVlbkh1ZT0iMCIKICAgY3JzOkdyZWVuU2F0dXJhdGlvbj0iMCIKICAgY3JzOkJsdWVIdWU9IjAiCiAgIGNyczpCbHVlU2F0dXJhdGlvbj0iMCIKICAgY3JzOkhEUkVkaXRNb2RlPSIwIgogICBjcnM6Q29udmVydFRvR3JheXNjYWxlPSJGYWxzZSIKICAgY3JzOk92ZXJyaWRlTG9va1ZpZ25ldHRlPSJGYWxzZSIKICAgY3JzOlRvbmVDdXJ2ZU5hbWUyMDEyPSJMaW5lYXIiCiAgIGNyczpDYW1lcmFQcm9maWxlPSJFbWJlZGRlZCIKICAgY3JzOkNhbWVyYVByb2ZpbGVEaWdlc3Q9IjU0NjUwQTM0MUI1QjVDQ0FFODQ0MkQwQjQzQTkyQkNFIgogICBjcnM6SGFzU2V0dGluZ3M9IlRydWUiCiAgIGNyczpDcm9wVG9wPSIwIgogICBjcnM6Q3JvcExlZnQ9IjAiCiAgIGNyczpDcm9wQm90dG9tPSIxIgogICBjcnM6Q3JvcFJpZ2h0PSIxIgogICBjcnM6Q3JvcEFuZ2xlPSIwIgogICBjcnM6Q3JvcENvbnN0cmFpblRvV2FycD0iMCIKICAgY3JzOkNyb3BDb25zdHJhaW5Ub1VuaXRTcXVhcmU9IjEiCiAgIGNyczpIYXNDcm9wPSJGYWxzZSIKICAgY3JzOkFscmVhZHlBcHBsaWVkPSJUcnVlIj4KICAgPHhtcE1NOkhpc3Rvcnk+CiAgICA8cmRmOlNlcT4KICAgICA8cmRmOmxpCiAgICAgIHN0RXZ0OmFjdGlvbj0iZGVyaXZlZCIKICAgICAgc3RFdnQ6cGFyYW1ldGVycz0ic2F2ZWQgdG8gbmV3IGxvY2F0aW9uIi8+CiAgICAgPHJkZjpsaQogICAgICBzdEV2dDphY3Rpb249InNhdmVkIgogICAgICBzdEV2dDppbnN0YW5jZUlEPSJ4bXAuaWlkOmY2NjczNjY2LWFhZDktNGFlNy04ZGNlLWYwMmUwODBiODNjMiIKICAgICAgc3RFdnQ6d2hlbj0iMjAyNi0wMS0zMVQwNDoxODowMSswNjowMCIKICAgICAgc3RFdnQ6c29mdHdhcmVBZ2VudD0iQWRvYmUgUGhvdG9zaG9wIExpZ2h0cm9vbSBDbGFzc2ljIDE1LjEuMSAoTWFjaW50b3NoKSIKICAgICAgc3RFdnQ6Y2hhbmdlZD0iLyIvPgogICAgIDxyZGY6bGkKICAgICAgc3RFdnQ6YWN0aW9uPSJkZXJpdmVkIgogICAgICBzdEV2dDpwYXJhbWV0ZXJzPSJjb252ZXJ0ZWQgZnJvbSBpbWFnZS9kbmcgdG8gaW1hZ2UvanBlZywgc2F2ZWQgdG8gbmV3IGxvY2F0aW9uIi8+CiAgICAgPHJkZjpsaQogICAgICBzdEV2dDphY3Rpb249InNhdmVkIgogICAgICBzdEV2dDppbnN0YW5jZUlEPSJ4bXAuaWlkOjIyOGY2NGFmLTJkYjgtNGFjZC1iNWVhLTQzOGIxZTI2MGVmZCIKICAgICAgc3RFdnQ6d2hlbj0iMjAyNi0wMi0wN1QwOTowMzo0NiswNjowMCIKICAgICAgc3RFdnQ6c29mdHdhcmVBZ2VudD0iQWRvYmUgUGhvdG9zaG9wIExpZ2h0cm9vbSBDbGFzc2ljIDE1LjEuMSAoTWFjaW50b3NoKSIKICAgICAgc3RFdnQ6Y2hhbmdlZD0iLyIvPgogICAgIDxyZGY6bGkKICAgICAgc3RFdnQ6YWN0aW9uPSJkZXJpdmVkIgogICAgICBzdEV2dDpwYXJhbWV0ZXJzPSJzYXZlZCB0byBuZXcgbG9jYXRpb24iLz4KICAgICA8cmRmOmxpCiAgICAgIHN0RXZ0OmFjdGlvbj0ic2F2ZWQiCiAgICAgIHN0RXZ0Omluc3RhbmNlSUQ9InhtcC5paWQ6NjQxNzg4YjItNDg2Yi00ZDkxLWFjMWEtNDI4NTE0ZDM3YjE5IgogICAgICBzdEV2dDp3aGVuPSIyMDI2LTAyLTEyVDA0OjExOjEwKzA2OjAwIgogICAgICBzdEV2dDpzb2Z0d2FyZUFnZW50PSJBZG9iZSBQaG90b3Nob3AgTGlnaHRyb29tIENsYXNzaWMgMTUuMS4xIChNYWNpbnRvc2gpIgogICAgICBzdEV2dDpjaGFuZ2VkPSIvIi8+CiAgICA8L3JkZjpTZXE+CiAgIDwveG1wTU06SGlzdG9yeT4KICAgPHhtcE1NOkRlcml2ZWRGcm9tCiAgICBzdFJlZjppbnN0YW5jZUlEPSJ4bXAuaWlkOjIyOGY2NGFmLTJkYjgtNGFjZC1iNWVhLTQzOGIxZTI2MGVmZCIKICAgIHN0UmVmOmRvY3VtZW50SUQ9InhtcC5kaWQ6MjI4ZjY0YWYtMmRiOC00YWNkLWI1ZWEtNDM4YjFlMjYwZWZkIgogICAgc3RSZWY6b3JpZ2luYWxEb2N1bWVudElEPSIzOEU2MEY4M0EyRDYyQkRDQzRCQTdEMTZEMkM1Q0QxOSIvPgogICA8Y3JzOlRvbmVDdXJ2ZVBWMjAxMj4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+MCwgMDwvcmRmOmxpPgogICAgIDxyZGY6bGk+MjU1LCAyNTU8L3JkZjpsaT4KICAgIDwvcmRmOlNlcT4KICAgPC9jcnM6VG9uZUN1cnZlUFYyMDEyPgogICA8Y3JzOlRvbmVDdXJ2ZVBWMjAxMlJlZD4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+MCwgMDwvcmRmOmxpPgogICAgIDxyZGY6bGk+MjU1LCAyNTU8L3JkZjpsaT4KICAgIDwvcmRmOlNlcT4KICAgPC9jcnM6VG9uZUN1cnZlUFYyMDEyUmVkPgogICA8Y3JzOlRvbmVDdXJ2ZVBWMjAxMkdyZWVuPgogICAgPHJkZjpTZXE+CiAgICAgPHJkZjpsaT4wLCAwPC9yZGY6bGk+CiAgICAgPHJkZjpsaT4yNTUsIDI1NTwvcmRmOmxpPgogICAgPC9yZGY6U2VxPgogICA8L2NyczpUb25lQ3VydmVQVjIwMTJHcmVlbj4KICAgPGNyczpUb25lQ3VydmVQVjIwMTJCbHVlPgogICAgPHJkZjpTZXE+CiAgICAgPHJkZjpsaT4wLCAwPC9yZGY6bGk+CiAgICAgPHJkZjpsaT4yNTUsIDI1NTwvcmRmOmxpPgogICAgPC9yZGY6U2VxPgogICA8L2NyczpUb25lQ3VydmVQVjIwMTJCbHVlPgogICA8Y3JzOlBvaW50Q29sb3JzPgogICAgPHJkZjpTZXE+CiAgICAgPHJkZjpsaT4tMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDAsIC0xLjAwMDAwMCwgLTEuMDAwMDAwLCAtMS4wMDAwMDA8L3JkZjpsaT4KICAgIDwvcmRmOlNlcT4KICAgPC9jcnM6UG9pbnRDb2xvcnM+CiAgIDxjcnM6Q29sb3JWYXJpYW5jZT4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+LTUwLjAwMDAwMDwvcmRmOmxpPgogICAgPC9yZGY6U2VxPgogICA8L2NyczpDb2xvclZhcmlhbmNlPgogICA8Y3JzOlJldG91Y2hBcmVhcz4KICAgIDxyZGY6U2VxPgogICAgIDxyZGY6bGk+CiAgICAgIDxyZGY6RGVzY3JpcHRpb24KICAgICAgIGNyczpTcG90VHlwZT0iY2xvbmUiCiAgICAgICBjcnM6U291cmNlU3RhdGU9InNvdXJjZUF1dG9Db21wdXRlZCIKICAgICAgIGNyczpNZXRob2Q9ImdhdXNzaWFuIgogICAgICAgY3JzOkhlYWxWZXJzaW9uPSIyIgogICAgICAgY3JzOlNvdXJjZVg9IjAuODAzMjQzIgogICAgICAgY3JzOk9mZnNldFk9IjAuNDEwODI0IgogICAgICAgY3JzOk9wYWNpdHk9IjEiCiAgICAgICBjcnM6RmVhdGhlcj0iMCIKICAgICAgIGNyczpTZWVkPSIyIj4KICAgICAgPGNyczpNYXNrcz4KICAgICAgIDxyZGY6U2VxPgogICAgICAgIDxyZGY6bGk+CiAgICAgICAgIDxyZGY6RGVzY3JpcHRpb24KICAgICAgICAgIGNyczpXaGF0PSJNYXNrL1BhaW50IgogICAgICAgICAgY3JzOk1hc2tBY3RpdmU9InRydWUiCiAgICAgICAgICBjcnM6TWFza0JsZW5kTW9kZT0iMCIKICAgICAgICAgIGNyczpNYXNrSW52ZXJ0ZWQ9ImZhbHNlIgogICAgICAgICAgY3JzOk1hc2tTeW5jSUQ9IkY2NURENTI0NTE1MzRDM0NBNjk1OTRCMjMxMjFGMzk4IgogICAgICAgICAgY3JzOk1hc2tWYWx1ZT0iMSIKICAgICAgICAgIGNyczpSYWRpdXM9IjAuMDAxODU1IgogICAgICAgICAgY3JzOkZsb3c9IjEiCiAgICAgICAgICBjcnM6Q2VudGVyV2VpZ2h0PSIxIj4KICAgICAgICAgPGNyczpEYWJzPgogICAgICAgICAgPHJkZjpTZXE+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA4MDA5IDAuNDEwODI0PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTk2IDAuNDExMzgwPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTg0IDAuNDExOTM1PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTcyIDAuNDEyNDkxPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3OTE1IDAuNDEzMDQxPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODgxIDAuNDEzNTk0PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODYzIDAuNDE0MTUwPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODU4IDAuNDE0NzA2PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODU4IDAuNDE1MjYyPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODU4IDAuNDE1ODE4PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA3ODgwIDAuNDE2MzczPC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA4MDI0IDAuNDE2ODg2PC9yZGY6bGk+CiAgICAgICAgICAgPHJkZjpsaT5kIDAuODA4MzgxIDAuNDE3MDM4PC</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Antonio Smith</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-06-19 15:36:57</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jonathan Morton</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>30583</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sycamore Manor</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>A-1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>time_log</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[{"start_date": "2026-06-19", "start_time": "10:36", "end_date": "", "end_time": "11:36"}]</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Antonio Smith</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-06-19 15:36:57</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Jonathan Morton</t>
         </is>

</xml_diff>